<commit_message>
NK41 i NKPXLH: nazwy w ofercie, 2500 kg z dopłatą wpisywaną w wycenie, KOB/GDW standardowo 0,5/2,5%, numer wersji
- oferta: NK41 (dawniej NKPXL/NKPXLT) i NKPXLH; migracja zapisanych szablonów
- wariant 2 na sztukę: pole Dopłata [zł/szt.] w wycenie; bez ceny wariant niedostępny,
  karta 'brak ceny' i opcja w ofercie pokazują komunikat
- KOB i GDW do zmiany w 'Stawki w tej wycenie' (w %); NK41 bez własnych stawek
- wersja programu na pulpicie i w kopii zapasowej

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -42,7 +42,7 @@
     <t>21.10.2026</t>
   </si>
   <si>
-    <t>Wygenerowano 21.10.2026, 19:25:59 · ceny netto w zł · szablon NKPXLH</t>
+    <t>Wygenerowano 22.10.2026, 08:15:57 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena ofertowa · zysk 28%</t>
@@ -102,7 +102,7 @@
     <t>Prześwit</t>
   </si>
   <si>
-    <t>18× NKPXL</t>
+    <t>18× NKPXLH</t>
   </si>
   <si>
     <t>340 cm</t>
@@ -171,7 +171,7 @@
     <t>Wariant 2500 kg</t>
   </si>
   <si>
-    <t>+700 USD/szt. do ceny urządzeń</t>
+    <t>+2702 zł/szt. do ceny urządzeń</t>
   </si>
   <si>
     <t>Konserwacja · wariant 1 · 18 szt.</t>

</xml_diff>

<commit_message>
Raport PDF wg komentarzy: bez paska negocjacji, nagłówki bez zalanego tła, dyskretne kafelki z ceną za MP równą cenie, układ agregatów w Wymiarach, dyskretna konserwacja (wersja 1.40)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="170">
   <si>
     <t>KALKULACJA NKPXLH</t>
   </si>
@@ -42,7 +42,7 @@
     <t>21.10.2026</t>
   </si>
   <si>
-    <t>Wygenerowano 27.10.2026, 12:24:44 · ceny netto w zł · szablon NKPXLH</t>
+    <t>Wygenerowano 27.10.2026, 14:03:05 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena ofertowa · zysk 28%</t>
@@ -126,12 +126,21 @@
     <t>Długość miejsca postojowego</t>
   </si>
   <si>
-    <t>3 szt. (3xA3)</t>
+    <t>3 szt.</t>
   </si>
   <si>
     <t>500 cm</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>Układ agregatów</t>
+  </si>
+  <si>
+    <t>3xA3</t>
+  </si>
+  <si>
     <t>Opis wariantu</t>
   </si>
   <si>
@@ -421,9 +430,6 @@
   </si>
   <si>
     <t>Pomarańczowe = zmienione względem domyślnego NK38</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>FEU</t>
@@ -1350,7 +1356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1889,166 +1895,166 @@
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="33" t="s">
+    <row r="37" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="B38" s="34" t="s">
+      <c r="B37" s="30"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="C38" s="34"/>
-      <c r="D38" s="34"/>
-      <c r="E38" s="34"/>
-      <c r="F38" s="34"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="35" t="s">
+      <c r="E37" s="30"/>
+      <c r="F37" s="30"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B39" s="35"/>
-      <c r="C39" s="35" t="s">
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="D39" s="35"/>
-      <c r="E39" s="35" t="s">
+      <c r="B40" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="F39" s="35"/>
-    </row>
-    <row r="40" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="36" t="s">
+      <c r="C40" s="34"/>
+      <c r="D40" s="34"/>
+      <c r="E40" s="34"/>
+      <c r="F40" s="34"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="36"/>
-      <c r="C40" s="36" t="s">
+      <c r="B41" s="35"/>
+      <c r="C41" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="D40" s="36"/>
-      <c r="E40" s="36" t="s">
+      <c r="D41" s="35"/>
+      <c r="E41" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="F40" s="36"/>
-    </row>
-    <row r="42" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="11" t="s">
+      <c r="F41" s="35"/>
+    </row>
+    <row r="42" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="36"/>
+      <c r="C42" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="12" t="s">
+      <c r="D42" s="36"/>
+      <c r="E42" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="F42" s="12" t="s">
+      <c r="F42" s="36"/>
+    </row>
+    <row r="44" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="11" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="37" t="s">
+      <c r="B44" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B43" s="38" t="s">
+      <c r="C44" s="11"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C43" s="38"/>
-      <c r="D43" s="38"/>
-      <c r="E43" s="39">
+      <c r="F44" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="B45" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" s="38"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="39">
         <v>73496.74956521747</v>
       </c>
-      <c r="F43" s="39">
+      <c r="F45" s="39">
         <v>70688.85482517496</v>
       </c>
     </row>
-    <row r="45" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="40" t="s">
-        <v>48</v>
-      </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40" t="s">
-        <v>49</v>
-      </c>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-    </row>
-    <row r="46" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="41" t="s">
-        <v>50</v>
-      </c>
-      <c r="B46" s="41"/>
-      <c r="C46" s="41"/>
-      <c r="D46" s="41" t="s">
+    <row r="47" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="E46" s="41"/>
-      <c r="F46" s="41"/>
-    </row>
-    <row r="47" ht="17" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="42" t="s">
+      <c r="B47" s="40"/>
+      <c r="C47" s="40"/>
+      <c r="D47" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="B47" s="42"/>
-      <c r="C47" s="42"/>
-      <c r="D47" s="42" t="s">
+      <c r="E47" s="40"/>
+      <c r="F47" s="40"/>
+    </row>
+    <row r="48" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="E47" s="42"/>
-      <c r="F47" s="42"/>
-    </row>
-    <row r="48" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="43" t="s">
+      <c r="B48" s="41"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="B48" s="43"/>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43" t="s">
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+    </row>
+    <row r="49" ht="17" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-    </row>
-    <row r="50" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="10" t="s">
+      <c r="B49" s="42"/>
+      <c r="C49" s="42"/>
+      <c r="D49" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="44" t="s">
+      <c r="E49" s="42"/>
+      <c r="F49" s="42"/>
+    </row>
+    <row r="50" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="B51" s="45" t="s">
+      <c r="B50" s="43"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="C51" s="45"/>
-      <c r="D51" s="45"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="44" t="s">
+      <c r="E50" s="43"/>
+      <c r="F50" s="43"/>
+    </row>
+    <row r="52" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B52" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="C52" s="45"/>
-      <c r="D52" s="45"/>
-      <c r="E52" s="45"/>
-      <c r="F52" s="45"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="10"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="B53" s="45" t="s">
         <v>61</v>
-      </c>
-      <c r="B53" s="45" t="s">
-        <v>62</v>
       </c>
       <c r="C53" s="45"/>
       <c r="D53" s="45"/>
@@ -2057,10 +2063,10 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="B54" s="45" t="s">
         <v>63</v>
-      </c>
-      <c r="B54" s="45" t="s">
-        <v>64</v>
       </c>
       <c r="C54" s="45"/>
       <c r="D54" s="45"/>
@@ -2069,18 +2075,42 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="44" t="s">
+        <v>64</v>
+      </c>
+      <c r="B55" s="45" t="s">
         <v>65</v>
-      </c>
-      <c r="B55" s="45" t="s">
-        <v>66</v>
       </c>
       <c r="C55" s="45"/>
       <c r="D55" s="45"/>
       <c r="E55" s="45"/>
       <c r="F55" s="45"/>
     </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="44" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="C56" s="45"/>
+      <c r="D56" s="45"/>
+      <c r="E56" s="45"/>
+      <c r="F56" s="45"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="B57" s="45" t="s">
+        <v>69</v>
+      </c>
+      <c r="C57" s="45"/>
+      <c r="D57" s="45"/>
+      <c r="E57" s="45"/>
+      <c r="F57" s="45"/>
+    </row>
   </sheetData>
-  <mergeCells count="54">
+  <mergeCells count="58">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:D2"/>
@@ -2112,29 +2142,33 @@
     <mergeCell ref="D35:F35"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="D36:F36"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="D37:F37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B45:D45"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="D47:F47"/>
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="D48:F48"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B51:F51"/>
-    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="A52:F52"/>
     <mergeCell ref="B53:F53"/>
     <mergeCell ref="B54:F54"/>
     <mergeCell ref="B55:F55"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B57:F57"/>
   </mergeCells>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.55" header="0.25" footer="0.25"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="80" fitToWidth="1" fitToHeight="1"/>
@@ -2155,7 +2189,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -2164,7 +2198,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -2173,7 +2207,7 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -2182,10 +2216,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="44" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B5" s="45" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C5" s="45"/>
       <c r="D5" s="45"/>
@@ -2193,10 +2227,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="44" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C6" s="45"/>
       <c r="D6" s="45"/>
@@ -2204,10 +2238,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="44" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B7" s="45" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C7" s="45"/>
       <c r="D7" s="45"/>
@@ -2215,10 +2249,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="44" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="45"/>
@@ -2226,10 +2260,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="44" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="45"/>
@@ -2237,7 +2271,7 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -2246,23 +2280,23 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="47" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B12" s="47" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C12" s="47"/>
       <c r="D12" s="47"/>
       <c r="E12" s="48" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="49" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B13" s="50" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C13" s="50"/>
       <c r="D13" s="50"/>
@@ -2272,10 +2306,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="52" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C14" s="53"/>
       <c r="D14" s="53"/>
@@ -2285,10 +2319,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="49" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B15" s="50" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C15" s="50"/>
       <c r="D15" s="50"/>
@@ -2298,10 +2332,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="52" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C16" s="53"/>
       <c r="D16" s="53"/>
@@ -2311,10 +2345,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="49" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B17" s="50" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C17" s="50"/>
       <c r="D17" s="50"/>
@@ -2324,10 +2358,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="52" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C18" s="53"/>
       <c r="D18" s="53"/>
@@ -2340,7 +2374,7 @@
         <v>22</v>
       </c>
       <c r="B19" s="50" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C19" s="50"/>
       <c r="D19" s="50"/>
@@ -2350,10 +2384,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="52" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B20" s="53" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C20" s="53"/>
       <c r="D20" s="53"/>
@@ -2363,10 +2397,10 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="49" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B21" s="50" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C21" s="50"/>
       <c r="D21" s="50"/>
@@ -2376,10 +2410,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="52" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B22" s="53" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C22" s="53"/>
       <c r="D22" s="53"/>
@@ -2389,10 +2423,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="49" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B23" s="50" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C23" s="50"/>
       <c r="D23" s="50"/>
@@ -2402,10 +2436,10 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="52" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B24" s="53" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C24" s="53"/>
       <c r="D24" s="53"/>
@@ -2415,10 +2449,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="49" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B25" s="50" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C25" s="50"/>
       <c r="D25" s="50"/>
@@ -2428,10 +2462,10 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="52" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B26" s="53" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C26" s="53"/>
       <c r="D26" s="53"/>
@@ -2441,10 +2475,10 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="49" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B27" s="50" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C27" s="50"/>
       <c r="D27" s="50"/>
@@ -2454,10 +2488,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="52" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B28" s="53" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C28" s="53"/>
       <c r="D28" s="53"/>
@@ -2467,10 +2501,10 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="58" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B29" s="59" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C29" s="59"/>
       <c r="D29" s="59"/>
@@ -2480,10 +2514,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="52" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B30" s="53" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C30" s="53"/>
       <c r="D30" s="53"/>
@@ -2493,10 +2527,10 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="49" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B31" s="50" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C31" s="50"/>
       <c r="D31" s="50"/>
@@ -2506,10 +2540,10 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="52" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B32" s="53" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C32" s="53"/>
       <c r="D32" s="53"/>
@@ -2519,10 +2553,10 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="49" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B33" s="50" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C33" s="50"/>
       <c r="D33" s="50"/>
@@ -2532,10 +2566,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="52" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B34" s="53" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C34" s="53"/>
       <c r="D34" s="53"/>
@@ -2545,10 +2579,10 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="58" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B35" s="59" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C35" s="59"/>
       <c r="D35" s="59"/>
@@ -2558,10 +2592,10 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="58" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B36" s="59" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C36" s="59"/>
       <c r="D36" s="59"/>
@@ -2571,7 +2605,7 @@
     </row>
     <row r="37" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="46" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B37" s="46"/>
       <c r="C37" s="46"/>
@@ -2580,7 +2614,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
@@ -2589,182 +2623,182 @@
     </row>
     <row r="40" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="61" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B40" s="62" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="C40" s="63" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D40" s="63"/>
       <c r="E40" s="64" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="41" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="63" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B41" s="65">
         <v>130</v>
       </c>
       <c r="C41" s="63" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D41" s="63"/>
       <c r="E41" s="64" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="63" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B42" s="65">
         <v>45</v>
       </c>
       <c r="C42" s="63" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D42" s="63"/>
       <c r="E42" s="64" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="43" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="61" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B43" s="62" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="C43" s="63" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D43" s="63"/>
       <c r="E43" s="64" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="44" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="63" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B44" s="64" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C44" s="63" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D44" s="63"/>
       <c r="E44" s="64" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="45" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="61" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B45" s="62" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="C45" s="63" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D45" s="63"/>
       <c r="E45" s="64" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="63" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B46" s="64" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C46" s="63" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D46" s="63"/>
       <c r="E46" s="64" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="47" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="61" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B47" s="62" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="C47" s="63" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D47" s="63"/>
       <c r="E47" s="64" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="63" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B48" s="64" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C48" s="63" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D48" s="63"/>
       <c r="E48" s="64" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="63" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B49" s="64" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C49" s="61" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D49" s="61"/>
       <c r="E49" s="62" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="63" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B50" s="64" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C50" s="63" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D50" s="63"/>
       <c r="E50" s="64" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="51" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="63" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B51" s="64" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C51" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="D51"/>
       <c r="E51" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Raport: prześwit z oznaczeniem P (jak H1 przy zagłębieniu)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -42,7 +42,7 @@
     <t>21.10.2026</t>
   </si>
   <si>
-    <t>Wygenerowano 27.10.2026, 14:03:05 · ceny netto w zł · szablon NKPXLH</t>
+    <t>Wygenerowano 27.10.2026, 14:04:45 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena ofertowa · zysk 28%</t>
@@ -105,7 +105,7 @@
     <t>18× NKPXLH</t>
   </si>
   <si>
-    <t>340 cm</t>
+    <t>P 340 cm</t>
   </si>
   <si>
     <t>Razem</t>

</xml_diff>

<commit_message>
Raport: ceny (oferta, zejście, próg) jako zwykła tabelka; KOB / GDW obok układu agregatów (wersja 1.41)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="172">
   <si>
     <t>KALKULACJA NKPXLH</t>
   </si>
@@ -42,7 +42,7 @@
     <t>21.10.2026</t>
   </si>
   <si>
-    <t>Wygenerowano 27.10.2026, 14:04:45 · ceny netto w zł · szablon NKPXLH</t>
+    <t>Wygenerowano 27.10.2026, 14:13:52 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena ofertowa · zysk 28%</t>
@@ -139,6 +139,12 @@
   </si>
   <si>
     <t>3xA3</t>
+  </si>
+  <si>
+    <t>KOB / GDW</t>
+  </si>
+  <si>
+    <t>0,5% / 2,5%</t>
   </si>
   <si>
     <t>Opis wariantu</t>
@@ -1356,7 +1362,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1919,166 +1925,166 @@
       <c r="E38" s="32"/>
       <c r="F38" s="32"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="33" t="s">
+    <row r="39" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B39" s="30"/>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="34" t="s">
+      <c r="E39" s="30"/>
+      <c r="F39" s="30"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" s="32"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-      <c r="E40" s="34"/>
-      <c r="F40" s="34"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="35" t="s">
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="35"/>
-      <c r="C41" s="35" t="s">
+      <c r="B42" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35" t="s">
+      <c r="C42" s="34"/>
+      <c r="D42" s="34"/>
+      <c r="E42" s="34"/>
+      <c r="F42" s="34"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="F41" s="35"/>
-    </row>
-    <row r="42" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="36" t="s">
+      <c r="B43" s="35"/>
+      <c r="C43" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="36"/>
-      <c r="C42" s="36" t="s">
+      <c r="D43" s="35"/>
+      <c r="E43" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="D42" s="36"/>
-      <c r="E42" s="36" t="s">
+      <c r="F43" s="35"/>
+    </row>
+    <row r="44" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="F42" s="36"/>
-    </row>
-    <row r="44" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="11" t="s">
+      <c r="B44" s="36"/>
+      <c r="C44" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="D44" s="36"/>
+      <c r="E44" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="C44" s="11"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="12" t="s">
+      <c r="F44" s="36"/>
+    </row>
+    <row r="46" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="F44" s="12" t="s">
+      <c r="B46" s="11" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="37" t="s">
+      <c r="C46" s="11"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B45" s="38" t="s">
+      <c r="F46" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C45" s="38"/>
-      <c r="D45" s="38"/>
-      <c r="E45" s="39">
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" s="38"/>
+      <c r="D47" s="38"/>
+      <c r="E47" s="39">
         <v>73496.74956521747</v>
       </c>
-      <c r="F45" s="39">
+      <c r="F47" s="39">
         <v>70688.85482517496</v>
       </c>
     </row>
-    <row r="47" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="40" t="s">
-        <v>51</v>
-      </c>
-      <c r="B47" s="40"/>
-      <c r="C47" s="40"/>
-      <c r="D47" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="E47" s="40"/>
-      <c r="F47" s="40"/>
-    </row>
-    <row r="48" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="41" t="s">
+    <row r="49" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="B48" s="41"/>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41" t="s">
+      <c r="B49" s="40"/>
+      <c r="C49" s="40"/>
+      <c r="D49" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-    </row>
-    <row r="49" ht="17" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="42" t="s">
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
+    </row>
+    <row r="50" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="41" t="s">
         <v>55</v>
       </c>
-      <c r="B49" s="42"/>
-      <c r="C49" s="42"/>
-      <c r="D49" s="42" t="s">
+      <c r="B50" s="41"/>
+      <c r="C50" s="41"/>
+      <c r="D50" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="E49" s="42"/>
-      <c r="F49" s="42"/>
-    </row>
-    <row r="50" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="43" t="s">
+      <c r="E50" s="41"/>
+      <c r="F50" s="41"/>
+    </row>
+    <row r="51" ht="17" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="B50" s="43"/>
-      <c r="C50" s="43"/>
-      <c r="D50" s="43" t="s">
+      <c r="B51" s="42"/>
+      <c r="C51" s="42"/>
+      <c r="D51" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-    </row>
-    <row r="52" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="10" t="s">
+      <c r="E51" s="42"/>
+      <c r="F51" s="42"/>
+    </row>
+    <row r="52" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="43" t="s">
         <v>59</v>
       </c>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="44" t="s">
+      <c r="B52" s="43"/>
+      <c r="C52" s="43"/>
+      <c r="D52" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="B53" s="45" t="s">
+      <c r="E52" s="43"/>
+      <c r="F52" s="43"/>
+    </row>
+    <row r="54" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C53" s="45"/>
-      <c r="D53" s="45"/>
-      <c r="E53" s="45"/>
-      <c r="F53" s="45"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="44" t="s">
-        <v>62</v>
-      </c>
-      <c r="B54" s="45" t="s">
-        <v>63</v>
-      </c>
-      <c r="C54" s="45"/>
-      <c r="D54" s="45"/>
-      <c r="E54" s="45"/>
-      <c r="F54" s="45"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="10"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="10"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="44" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B55" s="45" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C55" s="45"/>
       <c r="D55" s="45"/>
@@ -2087,10 +2093,10 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="44" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B56" s="45" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C56" s="45"/>
       <c r="D56" s="45"/>
@@ -2099,18 +2105,42 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="44" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B57" s="45" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C57" s="45"/>
       <c r="D57" s="45"/>
       <c r="E57" s="45"/>
       <c r="F57" s="45"/>
     </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="B58" s="45" t="s">
+        <v>69</v>
+      </c>
+      <c r="C58" s="45"/>
+      <c r="D58" s="45"/>
+      <c r="E58" s="45"/>
+      <c r="F58" s="45"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="44" t="s">
+        <v>70</v>
+      </c>
+      <c r="B59" s="45" t="s">
+        <v>71</v>
+      </c>
+      <c r="C59" s="45"/>
+      <c r="D59" s="45"/>
+      <c r="E59" s="45"/>
+      <c r="F59" s="45"/>
+    </row>
   </sheetData>
-  <mergeCells count="58">
+  <mergeCells count="62">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:D2"/>
@@ -2146,29 +2176,33 @@
     <mergeCell ref="D37:F37"/>
     <mergeCell ref="A38:C38"/>
     <mergeCell ref="D38:F38"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B47:D47"/>
     <mergeCell ref="A49:C49"/>
     <mergeCell ref="D49:F49"/>
     <mergeCell ref="A50:C50"/>
     <mergeCell ref="D50:F50"/>
-    <mergeCell ref="A52:F52"/>
-    <mergeCell ref="B53:F53"/>
-    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="A54:F54"/>
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B56:F56"/>
     <mergeCell ref="B57:F57"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="B59:F59"/>
   </mergeCells>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.55" header="0.25" footer="0.25"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="80" fitToWidth="1" fitToHeight="1"/>
@@ -2189,7 +2223,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -2198,7 +2232,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -2207,7 +2241,7 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -2216,10 +2250,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="44" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B5" s="45" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C5" s="45"/>
       <c r="D5" s="45"/>
@@ -2227,10 +2261,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="44" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C6" s="45"/>
       <c r="D6" s="45"/>
@@ -2238,10 +2272,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="44" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B7" s="45" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C7" s="45"/>
       <c r="D7" s="45"/>
@@ -2249,10 +2283,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="44" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="45"/>
@@ -2260,10 +2294,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="44" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="45"/>
@@ -2271,7 +2305,7 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -2280,23 +2314,23 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="47" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B12" s="47" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C12" s="47"/>
       <c r="D12" s="47"/>
       <c r="E12" s="48" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="49" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B13" s="50" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C13" s="50"/>
       <c r="D13" s="50"/>
@@ -2306,10 +2340,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="52" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C14" s="53"/>
       <c r="D14" s="53"/>
@@ -2319,10 +2353,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="49" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B15" s="50" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C15" s="50"/>
       <c r="D15" s="50"/>
@@ -2332,10 +2366,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="52" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C16" s="53"/>
       <c r="D16" s="53"/>
@@ -2345,10 +2379,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="49" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B17" s="50" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C17" s="50"/>
       <c r="D17" s="50"/>
@@ -2358,10 +2392,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="52" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C18" s="53"/>
       <c r="D18" s="53"/>
@@ -2374,7 +2408,7 @@
         <v>22</v>
       </c>
       <c r="B19" s="50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C19" s="50"/>
       <c r="D19" s="50"/>
@@ -2384,10 +2418,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="52" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B20" s="53" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C20" s="53"/>
       <c r="D20" s="53"/>
@@ -2397,10 +2431,10 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="49" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B21" s="50" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C21" s="50"/>
       <c r="D21" s="50"/>
@@ -2410,10 +2444,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="52" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B22" s="53" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C22" s="53"/>
       <c r="D22" s="53"/>
@@ -2423,10 +2457,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="49" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B23" s="50" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C23" s="50"/>
       <c r="D23" s="50"/>
@@ -2436,10 +2470,10 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="52" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B24" s="53" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C24" s="53"/>
       <c r="D24" s="53"/>
@@ -2449,10 +2483,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="49" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B25" s="50" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C25" s="50"/>
       <c r="D25" s="50"/>
@@ -2462,10 +2496,10 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="52" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B26" s="53" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C26" s="53"/>
       <c r="D26" s="53"/>
@@ -2475,10 +2509,10 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="49" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B27" s="50" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C27" s="50"/>
       <c r="D27" s="50"/>
@@ -2488,10 +2522,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="52" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B28" s="53" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C28" s="53"/>
       <c r="D28" s="53"/>
@@ -2501,10 +2535,10 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="58" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B29" s="59" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C29" s="59"/>
       <c r="D29" s="59"/>
@@ -2514,10 +2548,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="52" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B30" s="53" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C30" s="53"/>
       <c r="D30" s="53"/>
@@ -2527,10 +2561,10 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="49" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B31" s="50" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C31" s="50"/>
       <c r="D31" s="50"/>
@@ -2540,10 +2574,10 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="52" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B32" s="53" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C32" s="53"/>
       <c r="D32" s="53"/>
@@ -2553,10 +2587,10 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="49" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B33" s="50" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C33" s="50"/>
       <c r="D33" s="50"/>
@@ -2566,10 +2600,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="52" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B34" s="53" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C34" s="53"/>
       <c r="D34" s="53"/>
@@ -2579,10 +2613,10 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="58" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B35" s="59" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C35" s="59"/>
       <c r="D35" s="59"/>
@@ -2592,10 +2626,10 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="58" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B36" s="59" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C36" s="59"/>
       <c r="D36" s="59"/>
@@ -2605,7 +2639,7 @@
     </row>
     <row r="37" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="46" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B37" s="46"/>
       <c r="C37" s="46"/>
@@ -2614,7 +2648,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
@@ -2623,148 +2657,148 @@
     </row>
     <row r="40" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="61" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B40" s="62" t="s">
         <v>34</v>
       </c>
       <c r="C40" s="63" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D40" s="63"/>
       <c r="E40" s="64" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="41" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="63" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B41" s="65">
         <v>130</v>
       </c>
       <c r="C41" s="63" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D41" s="63"/>
       <c r="E41" s="64" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="42" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="63" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B42" s="65">
         <v>45</v>
       </c>
       <c r="C42" s="63" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D42" s="63"/>
       <c r="E42" s="64" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="43" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="61" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B43" s="62" t="s">
         <v>34</v>
       </c>
       <c r="C43" s="63" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D43" s="63"/>
       <c r="E43" s="64" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="63" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B44" s="64" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C44" s="63" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D44" s="63"/>
       <c r="E44" s="64" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="45" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="61" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B45" s="62" t="s">
         <v>34</v>
       </c>
       <c r="C45" s="63" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D45" s="63"/>
       <c r="E45" s="64" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="46" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="63" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B46" s="64" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C46" s="63" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D46" s="63"/>
       <c r="E46" s="64" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="47" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="61" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B47" s="62" t="s">
         <v>34</v>
       </c>
       <c r="C47" s="63" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D47" s="63"/>
       <c r="E47" s="64" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="48" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="63" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B48" s="64" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C48" s="63" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D48" s="63"/>
       <c r="E48" s="64" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="49" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="63" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B49" s="64" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C49" s="61" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D49" s="61"/>
       <c r="E49" s="62" t="s">
@@ -2773,25 +2807,25 @@
     </row>
     <row r="50" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="63" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B50" s="64" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C50" s="63" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D50" s="63"/>
       <c r="E50" s="64" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="51" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="63" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B51" s="64" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C51" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Raport: konserwacja jako tabelka stawek 35–60 zł (stawki z wyceny pogrubione); nazwy pozycji bez adresów komórek Excela (wersja 1.42)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -42,7 +42,7 @@
     <t>21.10.2026</t>
   </si>
   <si>
-    <t>Wygenerowano 27.10.2026, 14:13:52 · ceny netto w zł · szablon NKPXLH</t>
+    <t>Wygenerowano 27.10.2026, 14:16:58 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena ofertowa · zysk 28%</t>
@@ -297,25 +297,25 @@
     <t>Kwota</t>
   </si>
   <si>
-    <t>Osobodni montażu (F50)</t>
+    <t>Osobodni montażu</t>
   </si>
   <si>
     <t>z cennika osobodni na urządzenie + utrudnienia</t>
   </si>
   <si>
-    <t>Tygodnie / dni montażu (B55)</t>
+    <t>Tygodnie / dni montażu</t>
   </si>
   <si>
     <t>tygodniowe wyjazdy ekipy</t>
   </si>
   <si>
-    <t>Osobodni podróży i rozładunku (G59)</t>
+    <t>Osobodni podróży i rozładunku</t>
   </si>
   <si>
     <t>pomiary, odbiory, rozładunek i dojazdy ekipy</t>
   </si>
   <si>
-    <t>Dni pracy ekipy (J39)</t>
+    <t>Dni pracy ekipy</t>
   </si>
   <si>
     <t>(osd montażu + podróży) ÷ 4 os.</t>
@@ -420,7 +420,7 @@
     <t>14% od robocizny (26 105 zł) i zysku z narzutem</t>
   </si>
   <si>
-    <t>Cena kontraktu, zysk 28% (K39)</t>
+    <t>Cena kontraktu, zysk 28%</t>
   </si>
   <si>
     <t>suma ÷ (1 − KOB − GDW − zysk) + podatek</t>

</xml_diff>

<commit_message>
Raport: agregaty jako suma z podziałem 3 kW / 6 kW w nawiasie
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -42,7 +42,7 @@
     <t>21.10.2026</t>
   </si>
   <si>
-    <t>Wygenerowano 27.10.2026, 14:20:07 · ceny netto w zł · szablon NKPXLH</t>
+    <t>Wygenerowano 27.10.2026, 14:21:22 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena ofertowa · zysk 28%</t>
@@ -126,7 +126,7 @@
     <t>Długość miejsca postojowego</t>
   </si>
   <si>
-    <t>3 szt.</t>
+    <t>3 szt. (3 kW / 6 kW: nie podano)</t>
   </si>
   <si>
     <t>500 cm</t>

</xml_diff>

<commit_message>
Domyślne KOB 0,515% i GDW 2,685% we wszystkich szablonach, z migracją zapisanych szablonów (wersja 1.44)
Testy zgodności ze starym Excelem liczą z jego stawkami 0,5% / 2,5%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -42,7 +42,7 @@
     <t>21.10.2026</t>
   </si>
   <si>
-    <t>Wygenerowano 27.10.2026, 14:21:22 · ceny netto w zł · szablon NKPXLH</t>
+    <t>Wygenerowano 27.10.2026, 14:28:47 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena ofertowa · zysk 28%</t>
@@ -54,13 +54,13 @@
     <t>Próg opłacalności · zysk 0%</t>
   </si>
   <si>
-    <t>10 492 zł / MP · 2423 € / MP</t>
-  </si>
-  <si>
-    <t>rabat −14 291 zł (−3,78%)</t>
-  </si>
-  <si>
-    <t>maks. rabat −117 979 zł (−31,24%)</t>
+    <t>10 525 zł / MP · 2431 € / MP</t>
+  </si>
+  <si>
+    <t>rabat −14 372 zł (−3,79%)</t>
+  </si>
+  <si>
+    <t>maks. rabat −118 564 zł (−31,29%)</t>
   </si>
   <si>
     <t>Pole do negocjacji: o ile można zejść z ceny (2000 kg)</t>
@@ -144,7 +144,7 @@
     <t>KOB / GDW</t>
   </si>
   <si>
-    <t>0,5% / 2,5%</t>
+    <t>0,52% / 2,69%</t>
   </si>
   <si>
     <t>Opis wariantu</t>
@@ -393,13 +393,13 @@
     <t>KOB</t>
   </si>
   <si>
-    <t>0,5% ceny przed podatkiem (358 739 zł)</t>
+    <t>0,52% ceny przed podatkiem (359 782 zł)</t>
   </si>
   <si>
     <t>GDW</t>
   </si>
   <si>
-    <t>2,5% ceny przed podatkiem</t>
+    <t>2,69% ceny przed podatkiem</t>
   </si>
   <si>
     <t>Zysk 28%</t>
@@ -411,7 +411,7 @@
     <t>Zysk z narzutem (zysk + GDW)</t>
   </si>
   <si>
-    <t>zysk 28% + GDW 2,5%</t>
+    <t>zysk 28% + GDW 2,69%</t>
   </si>
   <si>
     <t>Podatek</t>
@@ -1421,15 +1421,15 @@
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
-        <v>377712.0146768458</v>
+        <v>378892.57403020735</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7">
-        <v>363421.4034006092</v>
+        <v>364520.4828011145</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="8">
-        <v>259733.44240869896</v>
+        <v>260328.7602708647</v>
       </c>
       <c r="F6" s="8"/>
     </row>
@@ -1482,7 +1482,7 @@
         <v>0.28</v>
       </c>
       <c r="B11" s="14">
-        <v>377712.0146768458</v>
+        <v>378892.57403020735</v>
       </c>
       <c r="C11" s="14">
         <v>0</v>
@@ -1491,10 +1491,10 @@
         <v>0</v>
       </c>
       <c r="E11" s="14">
-        <v>109415.43242571017</v>
+        <v>110399.097185866</v>
       </c>
       <c r="F11" s="14">
-        <v>10492.00040769016</v>
+        <v>10524.793723061315</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1502,19 +1502,19 @@
         <v>0.26</v>
       </c>
       <c r="B12" s="17">
-        <v>366199.0151697932</v>
+        <v>367313.7027914014</v>
       </c>
       <c r="C12" s="17">
-        <v>-11512.999507052591</v>
+        <v>-11578.871238805936</v>
       </c>
       <c r="D12" s="18">
-        <v>-0.030480893007606917</v>
+        <v>-0.030559773488415758</v>
       </c>
       <c r="E12" s="17">
-        <v>99360.63166250705</v>
+        <v>100288.10589055905</v>
       </c>
       <c r="F12" s="17">
-        <v>10172.194865827589</v>
+        <v>10203.158410872262</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1522,19 +1522,19 @@
         <v>0.255</v>
       </c>
       <c r="B13" s="20">
-        <v>363421.4034006092</v>
+        <v>364520.4828011145</v>
       </c>
       <c r="C13" s="20">
-        <v>-14290.611276236596</v>
+        <v>-14372.091229092854</v>
       </c>
       <c r="D13" s="21">
-        <v>-0.0378346748870645</v>
+        <v>-0.03793183665813158</v>
       </c>
       <c r="E13" s="20">
-        <v>96934.82308676923</v>
+        <v>97848.98877584263</v>
       </c>
       <c r="F13" s="20">
-        <v>10095.038983350256</v>
+        <v>10125.568966697625</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1542,19 +1542,19 @@
         <v>0.24</v>
       </c>
       <c r="B14" s="23">
-        <v>355316.86495079834</v>
+        <v>356371.0332690135</v>
       </c>
       <c r="C14" s="23">
-        <v>-22395.14972604747</v>
+        <v>-22521.540761193843</v>
       </c>
       <c r="D14" s="24">
-        <v>-0.05929160009698871</v>
+        <v>-0.05944043854340176</v>
       </c>
       <c r="E14" s="23">
-        <v>89856.77888632877</v>
+        <v>90732.66356752171</v>
       </c>
       <c r="F14" s="23">
-        <v>9869.912915299954</v>
+        <v>9899.195368583709</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1562,19 +1562,19 @@
         <v>0.22</v>
       </c>
       <c r="B15" s="23">
-        <v>345015.0960768165</v>
+        <v>346013.53323980136</v>
       </c>
       <c r="C15" s="23">
-        <v>-32696.918600029312</v>
+        <v>-32879.040790406</v>
       </c>
       <c r="D15" s="24">
-        <v>-0.08656573614160352</v>
+        <v>-0.08677668300721224</v>
       </c>
       <c r="E15" s="23">
-        <v>80859.79825821333</v>
+        <v>81688.20746496765</v>
       </c>
       <c r="F15" s="23">
-        <v>9583.752668800458</v>
+        <v>9611.487034438927</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1582,19 +1582,19 @@
         <v>0.2</v>
       </c>
       <c r="B16" s="23">
-        <v>335248.48402745713</v>
+        <v>336195.4863371107</v>
       </c>
       <c r="C16" s="23">
-        <v>-42463.530649388675</v>
+        <v>-42697.08769309666</v>
       </c>
       <c r="D16" s="24">
-        <v>-0.11242303395013434</v>
+        <v>-0.11268916473853251</v>
       </c>
       <c r="E16" s="23">
-        <v>72330.19324714286</v>
+        <v>73114.81678442161</v>
       </c>
       <c r="F16" s="23">
-        <v>9312.457889651587</v>
+        <v>9338.763509364186</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1602,19 +1602,19 @@
         <v>0.18</v>
       </c>
       <c r="B17" s="23">
-        <v>325976.38398059696</v>
+        <v>326875.817449785</v>
       </c>
       <c r="C17" s="23">
-        <v>-51735.630696248845</v>
+        <v>-52016.75658042234</v>
       </c>
       <c r="D17" s="24">
-        <v>-0.13697110148987882</v>
+        <v>-0.13728629206724777</v>
       </c>
       <c r="E17" s="23">
-        <v>64232.46697081012</v>
+        <v>64976.62360034999</v>
       </c>
       <c r="F17" s="23">
-        <v>9054.899555016582</v>
+        <v>9079.883818049584</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1622,19 +1622,19 @@
         <v>0.16</v>
       </c>
       <c r="B18" s="23">
-        <v>317162.1654175323</v>
+        <v>318017.5183093567</v>
       </c>
       <c r="C18" s="23">
-        <v>-60549.84925931349</v>
+        <v>-60875.05572085065</v>
       </c>
       <c r="D18" s="24">
-        <v>-0.16030691878074713</v>
+        <v>-0.16066573982523438</v>
       </c>
       <c r="E18" s="23">
-        <v>56534.62841182715</v>
+        <v>57241.311266975004</v>
       </c>
       <c r="F18" s="23">
-        <v>8810.060150487008</v>
+        <v>8833.819953037686</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1642,19 +1642,19 @@
         <v>0.14</v>
       </c>
       <c r="B19" s="23">
-        <v>308772.72847196483</v>
+        <v>309587.1563254708</v>
       </c>
       <c r="C19" s="23">
-        <v>-68939.28620488098</v>
+        <v>-69305.41770473658</v>
       </c>
       <c r="D19" s="24">
-        <v>-0.18251811837085052</v>
+        <v>-0.18291574566254545</v>
       </c>
       <c r="E19" s="23">
-        <v>49207.77002436145</v>
+        <v>49879.68551975338</v>
       </c>
       <c r="F19" s="23">
-        <v>8577.020235332357</v>
+        <v>8599.643231263077</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1662,19 +1662,19 @@
         <v>0.12</v>
       </c>
       <c r="B20" s="23">
-        <v>300778.08855912986</v>
+        <v>301554.45292573044</v>
       </c>
       <c r="C20" s="23">
-        <v>-76933.92611771595</v>
+        <v>-77338.12110447692</v>
       </c>
       <c r="D20" s="24">
-        <v>-0.2036840850390669</v>
+        <v>-0.20411622292262477</v>
       </c>
       <c r="E20" s="23">
-        <v>42225.70497277647</v>
+        <v>42865.30627004221</v>
       </c>
       <c r="F20" s="23">
-        <v>8354.946904420274</v>
+        <v>8376.51258127029</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1682,19 +1682,19 @@
         <v>0.1</v>
       </c>
       <c r="B21" s="23">
-        <v>293151.01829745976</v>
+        <v>293891.9201895726</v>
       </c>
       <c r="C21" s="23">
-        <v>-84560.99637938605</v>
+        <v>-85000.65384063474</v>
       </c>
       <c r="D21" s="24">
-        <v>-0.2238769038144916</v>
+        <v>-0.22433971966380642</v>
       </c>
       <c r="E21" s="23">
-        <v>35564.65440632184</v>
+        <v>36174.170303727886</v>
       </c>
       <c r="F21" s="23">
-        <v>8143.083841596104</v>
+        <v>8163.664449710351</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1702,19 +1702,19 @@
         <v>0.08</v>
       </c>
       <c r="B22" s="23">
-        <v>285866.7377104715</v>
+        <v>286574.5465856741</v>
       </c>
       <c r="C22" s="23">
-        <v>-91845.27696637431</v>
+        <v>-92318.02744453325</v>
       </c>
       <c r="D22" s="24">
-        <v>-0.24316218017304317</v>
+        <v>-0.24365224808331334</v>
       </c>
       <c r="E22" s="23">
-        <v>29202.97689903371</v>
+        <v>29784.436858418692</v>
       </c>
       <c r="F22" s="23">
-        <v>7940.742714179763</v>
+        <v>7960.40407182428</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1722,19 +1722,19 @@
         <v>0.06</v>
       </c>
       <c r="B23" s="23">
-        <v>278902.645281153</v>
+        <v>279579.52424185927</v>
       </c>
       <c r="C23" s="23">
-        <v>-98809.36939569283</v>
+        <v>-99313.04978834809</v>
       </c>
       <c r="D23" s="24">
-        <v>-0.261599752076274</v>
+        <v>-0.2621140043257494</v>
       </c>
       <c r="E23" s="23">
-        <v>23120.933567890108</v>
+        <v>23676.189467968943</v>
       </c>
       <c r="F23" s="23">
-        <v>7747.29570225425</v>
+        <v>7766.097895607202</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1742,19 +1742,19 @@
         <v>0.04</v>
       </c>
       <c r="B24" s="23">
-        <v>272238.08370900946</v>
+        <v>272886.01148182957</v>
       </c>
       <c r="C24" s="23">
-        <v>-105473.93096783635</v>
+        <v>-106006.56254837778</v>
       </c>
       <c r="D24" s="24">
-        <v>-0.27924431013420453</v>
+        <v>-0.279779995212908</v>
       </c>
       <c r="E24" s="23">
-        <v>17300.483498301077</v>
+        <v>17831.22860296961</v>
       </c>
       <c r="F24" s="23">
-        <v>7562.168991916929</v>
+        <v>7580.166985606377</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1762,19 +1762,19 @@
         <v>0.02</v>
       </c>
       <c r="B25" s="23">
-        <v>265854.13525569305</v>
+        <v>266474.92542053526</v>
       </c>
       <c r="C25" s="23">
-        <v>-111857.87942115276</v>
+        <v>-112417.64860967209</v>
       </c>
       <c r="D25" s="24">
-        <v>-0.2961459394318011</v>
+        <v>-0.29670058564069285</v>
       </c>
       <c r="E25" s="23">
-        <v>11725.105010589474</v>
+        <v>12232.89055927827</v>
       </c>
       <c r="F25" s="23">
-        <v>7384.837090435918</v>
+        <v>7402.081261681535</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1782,19 +1782,19 @@
         <v>0</v>
       </c>
       <c r="B26" s="26">
-        <v>259733.44240869896</v>
+        <v>260328.7602708647</v>
       </c>
       <c r="C26" s="26">
-        <v>-117978.57226814685</v>
+        <v>-118563.81375934265</v>
       </c>
       <c r="D26" s="27">
-        <v>-0.31235059432537315</v>
+        <v>-0.31292197811691636</v>
       </c>
       <c r="E26" s="26">
-        <v>6379.639037835052</v>
+        <v>6865.888798384091</v>
       </c>
       <c r="F26" s="26">
-        <v>7214.817844686082</v>
+        <v>7231.354451968464</v>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2015,10 +2015,10 @@
       <c r="C47" s="38"/>
       <c r="D47" s="38"/>
       <c r="E47" s="39">
-        <v>73496.74956521747</v>
+        <v>73728.71209883725</v>
       </c>
       <c r="F47" s="39">
-        <v>70688.85482517496</v>
+        <v>70904.8077475456</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2556,7 +2556,7 @@
       <c r="C30" s="53"/>
       <c r="D30" s="53"/>
       <c r="E30" s="57">
-        <v>1793.695613536232</v>
+        <v>1852.8771403200583</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -2569,7 +2569,7 @@
       <c r="C31" s="50"/>
       <c r="D31" s="50"/>
       <c r="E31" s="56">
-        <v>8968.47806768116</v>
+        <v>9660.145867493897</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -2582,7 +2582,7 @@
       <c r="C32" s="53"/>
       <c r="D32" s="53"/>
       <c r="E32" s="57">
-        <v>100446.954358029</v>
+        <v>100738.95131837211</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -2595,7 +2595,7 @@
       <c r="C33" s="50"/>
       <c r="D33" s="50"/>
       <c r="E33" s="56">
-        <v>109415.43242571017</v>
+        <v>110399.097185866</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -2608,7 +2608,7 @@
       <c r="C34" s="53"/>
       <c r="D34" s="53"/>
       <c r="E34" s="57">
-        <v>18972.891969599426</v>
+        <v>19110.605036021243</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -2621,7 +2621,7 @@
       <c r="C35" s="59"/>
       <c r="D35" s="59"/>
       <c r="E35" s="60">
-        <v>377712.0146768458</v>
+        <v>378892.57403020735</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -2634,7 +2634,7 @@
       <c r="C36" s="59"/>
       <c r="D36" s="59"/>
       <c r="E36" s="60">
-        <v>268296.5822511356</v>
+        <v>268493.4768443414</v>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Raport i Excel: data kalkulacji z godziną przygotowania raportu (wersja 1.47)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -39,10 +39,10 @@
     <t>ul. Kwiatowa 24, Piastów</t>
   </si>
   <si>
-    <t>21.10.2026</t>
-  </si>
-  <si>
-    <t>Wygenerowano 27.10.2026, 14:33:08 · ceny netto w zł · szablon NKPXLH</t>
+    <t>21.10.2026, 14:43</t>
+  </si>
+  <si>
+    <t>Wygenerowano 27.10.2026, 14:43:39 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena</t>

</xml_diff>

<commit_message>
Wycena łączona: drugie urządzenie w jednej kalkulacji (wspólna ekipa, osobne ceny pozycji)
Silnik sumuje materiały i osobodni obu urządzeń, wspólne koszty liczy raz
i dzieli cenę na pozycje wg osobodni. Formularz ma kartę Drugie urządzenie,
oferta Pozycję 2 z danymi technicznymi i ceną, raport i Excel obie pozycje.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -39,10 +39,10 @@
     <t>ul. Kwiatowa 24, Piastów</t>
   </si>
   <si>
-    <t>21.10.2026, 14:43</t>
-  </si>
-  <si>
-    <t>Wygenerowano 27.10.2026, 14:43:39 · ceny netto w zł · szablon NKPXLH</t>
+    <t>21.10.2026, 17:30</t>
+  </si>
+  <si>
+    <t>Wygenerowano 27.10.2026, 17:30:54 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena</t>
@@ -716,7 +716,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -766,6 +766,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="hair">
+        <color rgb="FFD3D9DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -946,13 +955,13 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
Excel: jeden arkusz, wydruk na 3 stronach (2 kartki dwustronnie)
Podsumowanie, koszty i cennik na wspólnej siatce 6 kolumn, osobna strona
dla każdej części; cennik nie wychodzi już poza stronę.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -4,29 +4,12 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Podsumowanie" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Obliczenia i cennik" state="visible" r:id="rId5"/>
+    <sheet sheetId="1" name="Kalkulacja" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="B41" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="B42" authorId="0">
-      <text/>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="175">
   <si>
@@ -39,10 +22,10 @@
     <t>ul. Kwiatowa 24, Piastów</t>
   </si>
   <si>
-    <t>21.10.2026, 10:10</t>
-  </si>
-  <si>
-    <t>Wygenerowano 30.10.2026, 10:10:16 · ceny netto w zł · szablon NKPXLH</t>
+    <t>21.10.2026, 10:28</t>
+  </si>
+  <si>
+    <t>Wygenerowano 30.10.2026, 10:28:00 · ceny netto w zł · szablon NKPXLH</t>
   </si>
   <si>
     <t>Cena</t>
@@ -222,6 +205,192 @@
     <t>60 zł / szt. / mies.</t>
   </si>
   <si>
+    <t>Koszty · 2000 kg · 28%</t>
+  </si>
+  <si>
+    <t>Skąd się biorą kwoty (wariant 2000 kg) · ceny netto w zł</t>
+  </si>
+  <si>
+    <t>Materiały i urządzenia</t>
+  </si>
+  <si>
+    <t>Urządzenia NKPXLH: 18 × 10901 zł (z frachtem 2023 zł/szt.)</t>
+  </si>
+  <si>
+    <t>196 215 zł</t>
+  </si>
+  <si>
+    <t>Fracht: kontener 36166 zł + ubezpieczenie 245 zł, × 1 kont. / 18 szt.</t>
+  </si>
+  <si>
+    <t>36 411 zł</t>
+  </si>
+  <si>
+    <t>Hydraulika PXL (140 + 65 + 29 EUR/szt.)</t>
+  </si>
+  <si>
+    <t>3648 zł</t>
+  </si>
+  <si>
+    <t>Suma 2000 kg</t>
+  </si>
+  <si>
+    <t>199 862 zł</t>
+  </si>
+  <si>
+    <t>Suma 2500 kg (+24,33%)</t>
+  </si>
+  <si>
+    <t>248 498 zł</t>
+  </si>
+  <si>
+    <t>Montaż, narzuty i cena</t>
+  </si>
+  <si>
+    <t>Pozycja</t>
+  </si>
+  <si>
+    <t>Skąd ta kwota</t>
+  </si>
+  <si>
+    <t>Kwota</t>
+  </si>
+  <si>
+    <t>Osobodni montażu</t>
+  </si>
+  <si>
+    <t>z cennika osobodni na urządzenie + utrudnienia</t>
+  </si>
+  <si>
+    <t>Tygodnie / dni montażu</t>
+  </si>
+  <si>
+    <t>tygodniowe wyjazdy ekipy</t>
+  </si>
+  <si>
+    <t>Osobodni podróży i rozładunku</t>
+  </si>
+  <si>
+    <t>pomiary, odbiory, rozładunek i dojazdy ekipy</t>
+  </si>
+  <si>
+    <t>Dni pracy ekipy</t>
+  </si>
+  <si>
+    <t>(osd montażu + podróży) ÷ 4 os.</t>
+  </si>
+  <si>
+    <t>Kilometry auta</t>
+  </si>
+  <si>
+    <t>dojazdy na montaż, pomiary i odbiory w obie strony</t>
+  </si>
+  <si>
+    <t>Noclegi (osobonoce)</t>
+  </si>
+  <si>
+    <t>(dni pracy + 1) × 4 os.</t>
+  </si>
+  <si>
+    <t>cena urządzeń i pozycji kosztowych (patrz wyżej)</t>
+  </si>
+  <si>
+    <t>Paliwo</t>
+  </si>
+  <si>
+    <t>4020 km × 113 zł/100 km (12 l × 9,4 zł)</t>
+  </si>
+  <si>
+    <t>Hotel</t>
+  </si>
+  <si>
+    <t>64 noclegów × 130 zł/doba</t>
+  </si>
+  <si>
+    <t>1 kont. × 3500 zł</t>
+  </si>
+  <si>
+    <t>Spider Crane</t>
+  </si>
+  <si>
+    <t>2 dni × 1200 zł/dzień</t>
+  </si>
+  <si>
+    <t>Rozładunek, sprzęt</t>
+  </si>
+  <si>
+    <t>2800 zł × 1 transp.</t>
+  </si>
+  <si>
+    <t>Rozładunek, ludzie</t>
+  </si>
+  <si>
+    <t>1 dni × 4 os. × 413 zł</t>
+  </si>
+  <si>
+    <t>Dojazdy, ludzie</t>
+  </si>
+  <si>
+    <t>17,06 osd podróży × 413 zł</t>
+  </si>
+  <si>
+    <t>36 osd × 413 zł (średnia stawka)</t>
+  </si>
+  <si>
+    <t>Diety</t>
+  </si>
+  <si>
+    <t>57,06 osd × 45 zł</t>
+  </si>
+  <si>
+    <t>Suma przed narzutami</t>
+  </si>
+  <si>
+    <t>suma kosztów powyżej</t>
+  </si>
+  <si>
+    <t>KOB</t>
+  </si>
+  <si>
+    <t>0,515% ceny przed podatkiem (359 782 zł)</t>
+  </si>
+  <si>
+    <t>GDW</t>
+  </si>
+  <si>
+    <t>2,685% ceny przed podatkiem</t>
+  </si>
+  <si>
+    <t>Zysk 28%</t>
+  </si>
+  <si>
+    <t>28% ceny przed podatkiem</t>
+  </si>
+  <si>
+    <t>Zysk z narzutem (zysk + GDW)</t>
+  </si>
+  <si>
+    <t>zysk 28% + GDW 2,685%</t>
+  </si>
+  <si>
+    <t>Podatek</t>
+  </si>
+  <si>
+    <t>14% od robocizny (26 105 zł) i zysku z narzutem</t>
+  </si>
+  <si>
+    <t>Cena kontraktu, zysk 28%</t>
+  </si>
+  <si>
+    <t>suma ÷ (1 − KOB − GDW − zysk) + podatek</t>
+  </si>
+  <si>
+    <t>Koszt rzeczywisty</t>
+  </si>
+  <si>
+    <t>cena − zysk z narzutem</t>
+  </si>
+  <si>
     <t>Pozostałe dane wejściowe</t>
   </si>
   <si>
@@ -255,196 +424,10 @@
     <t>4.33 / 3.86</t>
   </si>
   <si>
-    <t>Koszty · 2000 kg · 28%</t>
-  </si>
-  <si>
-    <t>Strona 1: obliczenia · strona 2: cennik szablonu NKPXLH</t>
-  </si>
-  <si>
-    <t>Materiały i urządzenia</t>
-  </si>
-  <si>
-    <t>Urządzenia NKPXLH: 18 × 10901 zł (z frachtem 2023 zł/szt.)</t>
-  </si>
-  <si>
-    <t>196 215 zł</t>
-  </si>
-  <si>
-    <t>Fracht: kontener 36166 zł + ubezpieczenie 245 zł, × 1 kont. / 18 szt.</t>
-  </si>
-  <si>
-    <t>36 411 zł</t>
-  </si>
-  <si>
-    <t>Hydraulika PXL (140 + 65 + 29 EUR/szt.)</t>
-  </si>
-  <si>
-    <t>3648 zł</t>
-  </si>
-  <si>
-    <t>Suma 2000 kg</t>
-  </si>
-  <si>
-    <t>199 862 zł</t>
-  </si>
-  <si>
-    <t>Suma 2500 kg (+24,33%)</t>
-  </si>
-  <si>
-    <t>248 498 zł</t>
-  </si>
-  <si>
-    <t>Montaż, narzuty i cena</t>
-  </si>
-  <si>
-    <t>Pozycja</t>
-  </si>
-  <si>
-    <t>Skąd ta kwota</t>
-  </si>
-  <si>
-    <t>Kwota</t>
-  </si>
-  <si>
-    <t>Osobodni montażu</t>
-  </si>
-  <si>
-    <t>z cennika osobodni na urządzenie + utrudnienia</t>
-  </si>
-  <si>
-    <t>Tygodnie / dni montażu</t>
-  </si>
-  <si>
-    <t>tygodniowe wyjazdy ekipy</t>
-  </si>
-  <si>
-    <t>Osobodni podróży i rozładunku</t>
-  </si>
-  <si>
-    <t>pomiary, odbiory, rozładunek i dojazdy ekipy</t>
-  </si>
-  <si>
-    <t>Dni pracy ekipy</t>
-  </si>
-  <si>
-    <t>(osd montażu + podróży) ÷ 4 os.</t>
-  </si>
-  <si>
-    <t>Kilometry auta</t>
-  </si>
-  <si>
-    <t>dojazdy na montaż, pomiary i odbiory w obie strony</t>
-  </si>
-  <si>
-    <t>Noclegi (osobonoce)</t>
-  </si>
-  <si>
-    <t>(dni pracy + 1) × 4 os.</t>
-  </si>
-  <si>
-    <t>cena urządzeń i pozycji kosztowych (patrz wyżej)</t>
-  </si>
-  <si>
-    <t>Paliwo</t>
-  </si>
-  <si>
-    <t>4020 km × 113 zł/100 km (12 l × 9,4 zł)</t>
-  </si>
-  <si>
-    <t>Hotel</t>
-  </si>
-  <si>
-    <t>64 noclegów × 130 zł/doba</t>
-  </si>
-  <si>
-    <t>1 kont. × 3500 zł</t>
-  </si>
-  <si>
-    <t>Spider Crane</t>
-  </si>
-  <si>
-    <t>2 dni × 1200 zł/dzień</t>
-  </si>
-  <si>
-    <t>Rozładunek, sprzęt</t>
-  </si>
-  <si>
-    <t>2800 zł × 1 transp.</t>
-  </si>
-  <si>
-    <t>Rozładunek, ludzie</t>
-  </si>
-  <si>
-    <t>1 dni × 4 os. × 413 zł</t>
-  </si>
-  <si>
-    <t>Dojazdy, ludzie</t>
-  </si>
-  <si>
-    <t>17,06 osd podróży × 413 zł</t>
-  </si>
-  <si>
-    <t>36 osd × 413 zł (średnia stawka)</t>
-  </si>
-  <si>
-    <t>Diety</t>
-  </si>
-  <si>
-    <t>57,06 osd × 45 zł</t>
-  </si>
-  <si>
-    <t>Suma przed narzutami</t>
-  </si>
-  <si>
-    <t>suma kosztów powyżej</t>
-  </si>
-  <si>
-    <t>KOB</t>
-  </si>
-  <si>
-    <t>0,515% ceny przed podatkiem (359 782 zł)</t>
-  </si>
-  <si>
-    <t>GDW</t>
-  </si>
-  <si>
-    <t>2,685% ceny przed podatkiem</t>
-  </si>
-  <si>
-    <t>Zysk 28%</t>
-  </si>
-  <si>
-    <t>28% ceny przed podatkiem</t>
-  </si>
-  <si>
-    <t>Zysk z narzutem (zysk + GDW)</t>
-  </si>
-  <si>
-    <t>zysk 28% + GDW 2,685%</t>
-  </si>
-  <si>
-    <t>Podatek</t>
-  </si>
-  <si>
-    <t>14% od robocizny (26 105 zł) i zysku z narzutem</t>
-  </si>
-  <si>
-    <t>Cena kontraktu, zysk 28%</t>
-  </si>
-  <si>
-    <t>suma ÷ (1 − KOB − GDW − zysk) + podatek</t>
-  </si>
-  <si>
-    <t>Koszt rzeczywisty</t>
-  </si>
-  <si>
-    <t>cena − zysk z narzutem</t>
-  </si>
-  <si>
     <t>Cennik szablonu NKPXLH</t>
   </si>
   <si>
-    <t>Pomarańczowe = zmienione względem domyślnego NK38</t>
+    <t>Pomarańczowe = zmienione względem domyślnego NKPXLH</t>
   </si>
   <si>
     <t>FEU</t>
@@ -779,7 +762,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom"/>
@@ -905,17 +888,17 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
@@ -956,13 +939,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment indent="1"/>
+      <alignment indent="3"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment indent="1"/>
+    </xf>
     <xf numFmtId="171" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment indent="3"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1303,7 +1292,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2098,78 +2087,740 @@
         <v>6480</v>
       </c>
     </row>
-    <row r="58" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="11" t="s">
+    <row r="58" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="B58" s="11"/>
-      <c r="C58" s="11"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="11"/>
-      <c r="F58" s="11"/>
+      <c r="B58" s="43"/>
+      <c r="C58" s="43"/>
+      <c r="D58" s="43"/>
+      <c r="E58" s="43"/>
+      <c r="F58" s="43"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="43" t="s">
+      <c r="A59" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="B59" s="44" t="s">
-        <v>66</v>
-      </c>
+      <c r="B59" s="44"/>
       <c r="C59" s="44"/>
       <c r="D59" s="44"/>
       <c r="E59" s="44"/>
       <c r="F59" s="44"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="43" t="s">
+    <row r="61" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B61" s="11"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="11"/>
+      <c r="E61" s="11"/>
+      <c r="F61" s="11"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="B60" s="44" t="s">
+      <c r="B62" s="45"/>
+      <c r="C62" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="C60" s="44"/>
-      <c r="D60" s="44"/>
-      <c r="E60" s="44"/>
-      <c r="F60" s="44"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="43" t="s">
+      <c r="D62" s="46"/>
+      <c r="E62" s="46"/>
+      <c r="F62" s="46"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="B61" s="44" t="s">
+      <c r="B63" s="45"/>
+      <c r="C63" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="C61" s="44"/>
-      <c r="D61" s="44"/>
-      <c r="E61" s="44"/>
-      <c r="F61" s="44"/>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="43" t="s">
+      <c r="D63" s="46"/>
+      <c r="E63" s="46"/>
+      <c r="F63" s="46"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="B62" s="44" t="s">
+      <c r="B64" s="45"/>
+      <c r="C64" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="C62" s="44"/>
-      <c r="D62" s="44"/>
-      <c r="E62" s="44"/>
-      <c r="F62" s="44"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="43" t="s">
+      <c r="D64" s="46"/>
+      <c r="E64" s="46"/>
+      <c r="F64" s="46"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="45" t="s">
         <v>73</v>
       </c>
-      <c r="B63" s="44" t="s">
+      <c r="B65" s="45"/>
+      <c r="C65" s="46" t="s">
         <v>74</v>
       </c>
-      <c r="C63" s="44"/>
-      <c r="D63" s="44"/>
-      <c r="E63" s="44"/>
-      <c r="F63" s="44"/>
+      <c r="D65" s="46"/>
+      <c r="E65" s="46"/>
+      <c r="F65" s="46"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="45" t="s">
+        <v>75</v>
+      </c>
+      <c r="B66" s="45"/>
+      <c r="C66" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="D66" s="46"/>
+      <c r="E66" s="46"/>
+      <c r="F66" s="46"/>
+    </row>
+    <row r="68" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B68" s="11"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="11"/>
+      <c r="F68" s="11"/>
+    </row>
+    <row r="69" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B69" s="6"/>
+      <c r="C69" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D69" s="6"/>
+      <c r="E69" s="6"/>
+      <c r="F69" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="47" t="s">
+        <v>81</v>
+      </c>
+      <c r="B70" s="47"/>
+      <c r="C70" s="48" t="s">
+        <v>82</v>
+      </c>
+      <c r="D70" s="48"/>
+      <c r="E70" s="48"/>
+      <c r="F70" s="49">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="50" t="s">
+        <v>83</v>
+      </c>
+      <c r="B71" s="50"/>
+      <c r="C71" s="51" t="s">
+        <v>84</v>
+      </c>
+      <c r="D71" s="51"/>
+      <c r="E71" s="51"/>
+      <c r="F71" s="52">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="47" t="s">
+        <v>85</v>
+      </c>
+      <c r="B72" s="47"/>
+      <c r="C72" s="48" t="s">
+        <v>86</v>
+      </c>
+      <c r="D72" s="48"/>
+      <c r="E72" s="48"/>
+      <c r="F72" s="49">
+        <v>21.0606</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="50" t="s">
+        <v>87</v>
+      </c>
+      <c r="B73" s="50"/>
+      <c r="C73" s="51" t="s">
+        <v>88</v>
+      </c>
+      <c r="D73" s="51"/>
+      <c r="E73" s="51"/>
+      <c r="F73" s="52">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="47" t="s">
+        <v>89</v>
+      </c>
+      <c r="B74" s="47"/>
+      <c r="C74" s="48" t="s">
+        <v>90</v>
+      </c>
+      <c r="D74" s="48"/>
+      <c r="E74" s="48"/>
+      <c r="F74" s="53">
+        <v>4020</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="50" t="s">
+        <v>91</v>
+      </c>
+      <c r="B75" s="50"/>
+      <c r="C75" s="51" t="s">
+        <v>92</v>
+      </c>
+      <c r="D75" s="51"/>
+      <c r="E75" s="51"/>
+      <c r="F75" s="52">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="B76" s="47"/>
+      <c r="C76" s="48" t="s">
+        <v>93</v>
+      </c>
+      <c r="D76" s="48"/>
+      <c r="E76" s="48"/>
+      <c r="F76" s="54">
+        <v>199862.17016799998</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="B77" s="50"/>
+      <c r="C77" s="51" t="s">
+        <v>95</v>
+      </c>
+      <c r="D77" s="51"/>
+      <c r="E77" s="51"/>
+      <c r="F77" s="55">
+        <v>4542.6</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="B78" s="47"/>
+      <c r="C78" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="D78" s="48"/>
+      <c r="E78" s="48"/>
+      <c r="F78" s="54">
+        <v>8320</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="50" t="s">
+        <v>44</v>
+      </c>
+      <c r="B79" s="50"/>
+      <c r="C79" s="51" t="s">
+        <v>98</v>
+      </c>
+      <c r="D79" s="51"/>
+      <c r="E79" s="51"/>
+      <c r="F79" s="55">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="47" t="s">
+        <v>99</v>
+      </c>
+      <c r="B80" s="47"/>
+      <c r="C80" s="48" t="s">
+        <v>100</v>
+      </c>
+      <c r="D80" s="48"/>
+      <c r="E80" s="48"/>
+      <c r="F80" s="54">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="50" t="s">
+        <v>101</v>
+      </c>
+      <c r="B81" s="50"/>
+      <c r="C81" s="51" t="s">
+        <v>102</v>
+      </c>
+      <c r="D81" s="51"/>
+      <c r="E81" s="51"/>
+      <c r="F81" s="55">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="B82" s="47"/>
+      <c r="C82" s="48" t="s">
+        <v>104</v>
+      </c>
+      <c r="D82" s="48"/>
+      <c r="E82" s="48"/>
+      <c r="F82" s="54">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="50" t="s">
+        <v>105</v>
+      </c>
+      <c r="B83" s="50"/>
+      <c r="C83" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="D83" s="51"/>
+      <c r="E83" s="51"/>
+      <c r="F83" s="55">
+        <v>7037.4975</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="B84" s="47"/>
+      <c r="C84" s="48" t="s">
+        <v>107</v>
+      </c>
+      <c r="D84" s="48"/>
+      <c r="E84" s="48"/>
+      <c r="F84" s="54">
+        <v>14850</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="50" t="s">
+        <v>108</v>
+      </c>
+      <c r="B85" s="50"/>
+      <c r="C85" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="D85" s="51"/>
+      <c r="E85" s="51"/>
+      <c r="F85" s="55">
+        <v>2567.727</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="56" t="s">
+        <v>110</v>
+      </c>
+      <c r="B86" s="56"/>
+      <c r="C86" s="57" t="s">
+        <v>111</v>
+      </c>
+      <c r="D86" s="57"/>
+      <c r="E86" s="57"/>
+      <c r="F86" s="58">
+        <v>247529.994668</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="50" t="s">
+        <v>112</v>
+      </c>
+      <c r="B87" s="50"/>
+      <c r="C87" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="D87" s="51"/>
+      <c r="E87" s="51"/>
+      <c r="F87" s="55">
+        <v>1852.8771403200583</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="47" t="s">
+        <v>114</v>
+      </c>
+      <c r="B88" s="47"/>
+      <c r="C88" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="D88" s="48"/>
+      <c r="E88" s="48"/>
+      <c r="F88" s="54">
+        <v>9660.145867493897</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="B89" s="50"/>
+      <c r="C89" s="51" t="s">
+        <v>117</v>
+      </c>
+      <c r="D89" s="51"/>
+      <c r="E89" s="51"/>
+      <c r="F89" s="55">
+        <v>100738.95131837211</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="47" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90" s="47"/>
+      <c r="C90" s="48" t="s">
+        <v>119</v>
+      </c>
+      <c r="D90" s="48"/>
+      <c r="E90" s="48"/>
+      <c r="F90" s="54">
+        <v>110399.097185866</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" s="50" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91" s="50"/>
+      <c r="C91" s="51" t="s">
+        <v>121</v>
+      </c>
+      <c r="D91" s="51"/>
+      <c r="E91" s="51"/>
+      <c r="F91" s="55">
+        <v>19110.605036021243</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="56" t="s">
+        <v>122</v>
+      </c>
+      <c r="B92" s="56"/>
+      <c r="C92" s="57" t="s">
+        <v>123</v>
+      </c>
+      <c r="D92" s="57"/>
+      <c r="E92" s="57"/>
+      <c r="F92" s="58">
+        <v>378892.57403020735</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" s="56" t="s">
+        <v>124</v>
+      </c>
+      <c r="B93" s="56"/>
+      <c r="C93" s="57" t="s">
+        <v>125</v>
+      </c>
+      <c r="D93" s="57"/>
+      <c r="E93" s="57"/>
+      <c r="F93" s="58">
+        <v>268493.4768443414</v>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B95" s="11"/>
+      <c r="C95" s="11"/>
+      <c r="D95" s="11"/>
+      <c r="E95" s="11"/>
+      <c r="F95" s="11"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" s="45" t="s">
+        <v>127</v>
+      </c>
+      <c r="B96" s="45"/>
+      <c r="C96" s="46" t="s">
+        <v>128</v>
+      </c>
+      <c r="D96" s="46"/>
+      <c r="E96" s="46"/>
+      <c r="F96" s="46"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" s="45" t="s">
+        <v>129</v>
+      </c>
+      <c r="B97" s="45"/>
+      <c r="C97" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="D97" s="46"/>
+      <c r="E97" s="46"/>
+      <c r="F97" s="46"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="B98" s="45"/>
+      <c r="C98" s="46" t="s">
+        <v>132</v>
+      </c>
+      <c r="D98" s="46"/>
+      <c r="E98" s="46"/>
+      <c r="F98" s="46"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" s="45" t="s">
+        <v>133</v>
+      </c>
+      <c r="B99" s="45"/>
+      <c r="C99" s="46" t="s">
+        <v>134</v>
+      </c>
+      <c r="D99" s="46"/>
+      <c r="E99" s="46"/>
+      <c r="F99" s="46"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" s="45" t="s">
+        <v>135</v>
+      </c>
+      <c r="B100" s="45"/>
+      <c r="C100" s="46" t="s">
+        <v>136</v>
+      </c>
+      <c r="D100" s="46"/>
+      <c r="E100" s="46"/>
+      <c r="F100" s="46"/>
+    </row>
+    <row r="102" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B102" s="43"/>
+      <c r="C102" s="43"/>
+      <c r="D102" s="43"/>
+      <c r="E102" s="43"/>
+      <c r="F102" s="43"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="B103" s="44"/>
+      <c r="C103" s="44"/>
+      <c r="D103" s="44"/>
+      <c r="E103" s="44"/>
+      <c r="F103" s="44"/>
+    </row>
+    <row r="105" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" s="59" t="s">
+        <v>43</v>
+      </c>
+      <c r="B105" s="60" t="s">
+        <v>35</v>
+      </c>
+      <c r="C105" s="61" t="s">
+        <v>139</v>
+      </c>
+      <c r="D105" s="61"/>
+      <c r="E105" s="61"/>
+      <c r="F105" s="62" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="106" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" s="63" t="s">
+        <v>141</v>
+      </c>
+      <c r="B106" s="64">
+        <v>130</v>
+      </c>
+      <c r="C106" s="61" t="s">
+        <v>142</v>
+      </c>
+      <c r="D106" s="61"/>
+      <c r="E106" s="61"/>
+      <c r="F106" s="62" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="107" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" s="63" t="s">
+        <v>144</v>
+      </c>
+      <c r="B107" s="64">
+        <v>45</v>
+      </c>
+      <c r="C107" s="61" t="s">
+        <v>145</v>
+      </c>
+      <c r="D107" s="61"/>
+      <c r="E107" s="61"/>
+      <c r="F107" s="62" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="108" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" s="59" t="s">
+        <v>147</v>
+      </c>
+      <c r="B108" s="60" t="s">
+        <v>35</v>
+      </c>
+      <c r="C108" s="61" t="s">
+        <v>148</v>
+      </c>
+      <c r="D108" s="61"/>
+      <c r="E108" s="61"/>
+      <c r="F108" s="62" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="109" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" s="63" t="s">
+        <v>150</v>
+      </c>
+      <c r="B109" s="62" t="s">
+        <v>151</v>
+      </c>
+      <c r="C109" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="D109" s="61"/>
+      <c r="E109" s="61"/>
+      <c r="F109" s="62" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="110" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" s="59" t="s">
+        <v>154</v>
+      </c>
+      <c r="B110" s="60" t="s">
+        <v>35</v>
+      </c>
+      <c r="C110" s="61" t="s">
+        <v>155</v>
+      </c>
+      <c r="D110" s="61"/>
+      <c r="E110" s="61"/>
+      <c r="F110" s="62" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="111" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" s="63" t="s">
+        <v>71</v>
+      </c>
+      <c r="B111" s="62" t="s">
+        <v>157</v>
+      </c>
+      <c r="C111" s="61" t="s">
+        <v>158</v>
+      </c>
+      <c r="D111" s="61"/>
+      <c r="E111" s="61"/>
+      <c r="F111" s="62" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="112" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" s="59" t="s">
+        <v>159</v>
+      </c>
+      <c r="B112" s="60" t="s">
+        <v>35</v>
+      </c>
+      <c r="C112" s="61" t="s">
+        <v>160</v>
+      </c>
+      <c r="D112" s="61"/>
+      <c r="E112" s="61"/>
+      <c r="F112" s="62" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="113" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="B113" s="62" t="s">
+        <v>163</v>
+      </c>
+      <c r="C113" s="61" t="s">
+        <v>164</v>
+      </c>
+      <c r="D113" s="61"/>
+      <c r="E113" s="61"/>
+      <c r="F113" s="62" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="114" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" s="63" t="s">
+        <v>166</v>
+      </c>
+      <c r="B114" s="62" t="s">
+        <v>167</v>
+      </c>
+      <c r="C114" s="65" t="s">
+        <v>168</v>
+      </c>
+      <c r="D114" s="65"/>
+      <c r="E114" s="65"/>
+      <c r="F114" s="60" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="115" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" s="63" t="s">
+        <v>169</v>
+      </c>
+      <c r="B115" s="62" t="s">
+        <v>170</v>
+      </c>
+      <c r="C115" s="61" t="s">
+        <v>171</v>
+      </c>
+      <c r="D115" s="61"/>
+      <c r="E115" s="61"/>
+      <c r="F115" s="62" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="116" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" s="63" t="s">
+        <v>173</v>
+      </c>
+      <c r="B116" s="62" t="s">
+        <v>174</v>
+      </c>
+      <c r="C116" t="s">
+        <v>35</v>
+      </c>
+      <c r="D116"/>
+      <c r="E116"/>
+      <c r="F116" t="s">
+        <v>35</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="56">
+  <mergeCells count="139">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:D2"/>
@@ -2221,702 +2872,103 @@
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="A56:C56"/>
     <mergeCell ref="A58:F58"/>
-    <mergeCell ref="B59:F59"/>
-    <mergeCell ref="B60:F60"/>
-    <mergeCell ref="B61:F61"/>
-    <mergeCell ref="B62:F62"/>
-    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="C62:F62"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="C63:F63"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="C64:F64"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="C65:F65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="C66:F66"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="A79:B79"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="A80:B80"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="A82:B82"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="A83:B83"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="A84:B84"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="A86:B86"/>
+    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="C87:E87"/>
+    <mergeCell ref="A88:B88"/>
+    <mergeCell ref="C88:E88"/>
+    <mergeCell ref="A89:B89"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="A91:B91"/>
+    <mergeCell ref="C91:E91"/>
+    <mergeCell ref="A92:B92"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="A93:B93"/>
+    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="A95:F95"/>
+    <mergeCell ref="A96:B96"/>
+    <mergeCell ref="C96:F96"/>
+    <mergeCell ref="A97:B97"/>
+    <mergeCell ref="C97:F97"/>
+    <mergeCell ref="A98:B98"/>
+    <mergeCell ref="C98:F98"/>
+    <mergeCell ref="A99:B99"/>
+    <mergeCell ref="C99:F99"/>
+    <mergeCell ref="A100:B100"/>
+    <mergeCell ref="C100:F100"/>
+    <mergeCell ref="A102:F102"/>
+    <mergeCell ref="A103:F103"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="C106:E106"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="C115:E115"/>
+    <mergeCell ref="C116:E116"/>
   </mergeCells>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.55" header="0.25" footer="0.25"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="80" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="78" fitToWidth="1" fitToHeight="1"/>
   <headerFooter>
     <oddFooter>&amp;L&amp;8ul. Kwiatowa 24, Piastów&amp;R&amp;8Strona &amp;P z &amp;N</oddFooter>
   </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E51"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="5" width="19" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
-        <v>76</v>
-      </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" s="44" t="s">
-        <v>79</v>
-      </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="43" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="43" t="s">
-        <v>82</v>
-      </c>
-      <c r="B7" s="44" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" s="44" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="43" t="s">
-        <v>86</v>
-      </c>
-      <c r="B9" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="47" t="s">
-        <v>92</v>
-      </c>
-      <c r="B13" s="48" t="s">
-        <v>93</v>
-      </c>
-      <c r="C13" s="48"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="49">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="50" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" s="51" t="s">
-        <v>95</v>
-      </c>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="52">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" s="48" t="s">
-        <v>97</v>
-      </c>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="49">
-        <v>21.0606</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="50" t="s">
-        <v>98</v>
-      </c>
-      <c r="B16" s="51" t="s">
-        <v>99</v>
-      </c>
-      <c r="C16" s="51"/>
-      <c r="D16" s="51"/>
-      <c r="E16" s="52">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="47" t="s">
-        <v>100</v>
-      </c>
-      <c r="B17" s="48" t="s">
-        <v>101</v>
-      </c>
-      <c r="C17" s="48"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="53">
-        <v>4020</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="50" t="s">
-        <v>102</v>
-      </c>
-      <c r="B18" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="C18" s="51"/>
-      <c r="D18" s="51"/>
-      <c r="E18" s="52">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="47" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="48" t="s">
-        <v>104</v>
-      </c>
-      <c r="C19" s="48"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="54">
-        <v>199862.17016799998</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="50" t="s">
-        <v>105</v>
-      </c>
-      <c r="B20" s="51" t="s">
-        <v>106</v>
-      </c>
-      <c r="C20" s="51"/>
-      <c r="D20" s="51"/>
-      <c r="E20" s="55">
-        <v>4542.6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="47" t="s">
-        <v>107</v>
-      </c>
-      <c r="B21" s="48" t="s">
-        <v>108</v>
-      </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="54">
-        <v>8320</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="51" t="s">
-        <v>109</v>
-      </c>
-      <c r="C22" s="51"/>
-      <c r="D22" s="51"/>
-      <c r="E22" s="55">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="B23" s="48" t="s">
-        <v>111</v>
-      </c>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="54">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="50" t="s">
-        <v>112</v>
-      </c>
-      <c r="B24" s="51" t="s">
-        <v>113</v>
-      </c>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="55">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="47" t="s">
-        <v>114</v>
-      </c>
-      <c r="B25" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="54">
-        <v>1650</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="50" t="s">
-        <v>116</v>
-      </c>
-      <c r="B26" s="51" t="s">
-        <v>117</v>
-      </c>
-      <c r="C26" s="51"/>
-      <c r="D26" s="51"/>
-      <c r="E26" s="55">
-        <v>7037.4975</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="B27" s="48" t="s">
-        <v>118</v>
-      </c>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="54">
-        <v>14850</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="50" t="s">
-        <v>119</v>
-      </c>
-      <c r="B28" s="51" t="s">
-        <v>120</v>
-      </c>
-      <c r="C28" s="51"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="55">
-        <v>2567.727</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="56" t="s">
-        <v>121</v>
-      </c>
-      <c r="B29" s="57" t="s">
-        <v>122</v>
-      </c>
-      <c r="C29" s="57"/>
-      <c r="D29" s="57"/>
-      <c r="E29" s="58">
-        <v>247529.994668</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="50" t="s">
-        <v>123</v>
-      </c>
-      <c r="B30" s="51" t="s">
-        <v>124</v>
-      </c>
-      <c r="C30" s="51"/>
-      <c r="D30" s="51"/>
-      <c r="E30" s="55">
-        <v>1852.8771403200583</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="47" t="s">
-        <v>125</v>
-      </c>
-      <c r="B31" s="48" t="s">
-        <v>126</v>
-      </c>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="54">
-        <v>9660.145867493897</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="50" t="s">
-        <v>127</v>
-      </c>
-      <c r="B32" s="51" t="s">
-        <v>128</v>
-      </c>
-      <c r="C32" s="51"/>
-      <c r="D32" s="51"/>
-      <c r="E32" s="55">
-        <v>100738.95131837211</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="47" t="s">
-        <v>129</v>
-      </c>
-      <c r="B33" s="48" t="s">
-        <v>130</v>
-      </c>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="54">
-        <v>110399.097185866</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="B34" s="51" t="s">
-        <v>132</v>
-      </c>
-      <c r="C34" s="51"/>
-      <c r="D34" s="51"/>
-      <c r="E34" s="55">
-        <v>19110.605036021243</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="56" t="s">
-        <v>133</v>
-      </c>
-      <c r="B35" s="57" t="s">
-        <v>134</v>
-      </c>
-      <c r="C35" s="57"/>
-      <c r="D35" s="57"/>
-      <c r="E35" s="58">
-        <v>378892.57403020735</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="56" t="s">
-        <v>135</v>
-      </c>
-      <c r="B36" s="57" t="s">
-        <v>136</v>
-      </c>
-      <c r="C36" s="57"/>
-      <c r="D36" s="57"/>
-      <c r="E36" s="58">
-        <v>268493.4768443414</v>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="45" t="s">
-        <v>137</v>
-      </c>
-      <c r="B37" s="45"/>
-      <c r="C37" s="45"/>
-      <c r="D37" s="45"/>
-      <c r="E37" s="45"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="46" t="s">
-        <v>138</v>
-      </c>
-      <c r="B38" s="46"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-    </row>
-    <row r="40" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="59" t="s">
-        <v>43</v>
-      </c>
-      <c r="B40" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="C40" s="61" t="s">
-        <v>139</v>
-      </c>
-      <c r="D40" s="61"/>
-      <c r="E40" s="62" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="41" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="61" t="s">
-        <v>141</v>
-      </c>
-      <c r="B41" s="63">
-        <v>130</v>
-      </c>
-      <c r="C41" s="61" t="s">
-        <v>142</v>
-      </c>
-      <c r="D41" s="61"/>
-      <c r="E41" s="62" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="42" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="61" t="s">
-        <v>144</v>
-      </c>
-      <c r="B42" s="63">
-        <v>45</v>
-      </c>
-      <c r="C42" s="61" t="s">
-        <v>145</v>
-      </c>
-      <c r="D42" s="61"/>
-      <c r="E42" s="62" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="43" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="B43" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="C43" s="61" t="s">
-        <v>148</v>
-      </c>
-      <c r="D43" s="61"/>
-      <c r="E43" s="62" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="44" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="61" t="s">
-        <v>150</v>
-      </c>
-      <c r="B44" s="62" t="s">
-        <v>151</v>
-      </c>
-      <c r="C44" s="61" t="s">
-        <v>152</v>
-      </c>
-      <c r="D44" s="61"/>
-      <c r="E44" s="62" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="45" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="59" t="s">
-        <v>154</v>
-      </c>
-      <c r="B45" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="C45" s="61" t="s">
-        <v>155</v>
-      </c>
-      <c r="D45" s="61"/>
-      <c r="E45" s="62" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="46" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="61" t="s">
-        <v>82</v>
-      </c>
-      <c r="B46" s="62" t="s">
-        <v>157</v>
-      </c>
-      <c r="C46" s="61" t="s">
-        <v>158</v>
-      </c>
-      <c r="D46" s="61"/>
-      <c r="E46" s="62" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="47" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="59" t="s">
-        <v>159</v>
-      </c>
-      <c r="B47" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="C47" s="61" t="s">
-        <v>160</v>
-      </c>
-      <c r="D47" s="61"/>
-      <c r="E47" s="62" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="48" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="61" t="s">
-        <v>162</v>
-      </c>
-      <c r="B48" s="62" t="s">
-        <v>163</v>
-      </c>
-      <c r="C48" s="61" t="s">
-        <v>164</v>
-      </c>
-      <c r="D48" s="61"/>
-      <c r="E48" s="62" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="49" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="61" t="s">
-        <v>166</v>
-      </c>
-      <c r="B49" s="62" t="s">
-        <v>167</v>
-      </c>
-      <c r="C49" s="59" t="s">
-        <v>168</v>
-      </c>
-      <c r="D49" s="59"/>
-      <c r="E49" s="60" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="61" t="s">
-        <v>169</v>
-      </c>
-      <c r="B50" s="62" t="s">
-        <v>170</v>
-      </c>
-      <c r="C50" s="61" t="s">
-        <v>171</v>
-      </c>
-      <c r="D50" s="61"/>
-      <c r="E50" s="62" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="51" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="61" t="s">
-        <v>173</v>
-      </c>
-      <c r="B51" s="62" t="s">
-        <v>174</v>
-      </c>
-      <c r="C51" t="s">
-        <v>35</v>
-      </c>
-      <c r="D51"/>
-      <c r="E51" t="s">
-        <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="48">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C51:D51"/>
-  </mergeCells>
-  <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.55" header="0.25" footer="0.25"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="82" fitToWidth="1" fitToHeight="1"/>
-  <headerFooter>
-    <oddFooter>&amp;L&amp;8ul. Kwiatowa 24, Piastów&amp;R&amp;8Strona &amp;P z &amp;N</oddFooter>
-  </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="36" max="16838" man="1"/>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="57" max="16838" man="1"/>
+    <brk id="101" max="16838" man="1"/>
   </rowBreaks>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Excel: strona 1 jak raport PDF (czcionka, ramki Zakres/Wymiary, układ cen)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Kwiatowa_24_Piastow_NKPXLH.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="176">
   <si>
     <t>KALKULACJA NKPXLH</t>
   </si>
@@ -22,10 +22,10 @@
     <t>ul. Kwiatowa 24, Piastów</t>
   </si>
   <si>
-    <t>21.10.2026, 12:42</t>
-  </si>
-  <si>
-    <t>Wygenerowano 30.10.2026, 12:42:34 · ceny netto w zł · szablon NKPXLH</t>
+    <t>21.10.2026, 12:45</t>
+  </si>
+  <si>
+    <t>Ceny netto · wygenerowano 30.10.2026</t>
   </si>
   <si>
     <t>Cena</t>
@@ -40,7 +40,10 @@
     <t>Rabat od oferty</t>
   </si>
   <si>
-    <t>Cena ofertowa · zysk 28% · 2000 kg · 2431 € / MP</t>
+    <t>Cena ofertowa · zysk 28% · 2000 kg</t>
+  </si>
+  <si>
+    <t>10 525 zł · 2431 €</t>
   </si>
   <si>
     <t>–</t>
@@ -52,13 +55,13 @@
     <t>−14 372 zł (−3,79%)</t>
   </si>
   <si>
-    <t>Próg opłacalności · zysk 0% (maks. rabat)</t>
+    <t>Próg opłacalności · zysk 0% · maks. rabat</t>
   </si>
   <si>
     <t>−118 564 zł (−31,29%)</t>
   </si>
   <si>
-    <t>Pole do negocjacji: o ile można zejść z ceny (2000 kg)</t>
+    <t>Pole do negocjacji (2000 kg)</t>
   </si>
   <si>
     <t>Zysk</t>
@@ -124,10 +127,10 @@
     <t>Układ agregatów</t>
   </si>
   <si>
+    <t>KOB / GDW</t>
+  </si>
+  <si>
     <t>3xA3</t>
-  </si>
-  <si>
-    <t>KOB / GDW</t>
   </si>
   <si>
     <t>0,515% / 2,685%</t>
@@ -552,7 +555,7 @@
     <numFmt numFmtId="170" formatCode="&quot;+&quot;#,##0 &quot;zł&quot;"/>
     <numFmt numFmtId="171" formatCode="#,##0.##"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -562,98 +565,104 @@
     </font>
     <font>
       <color rgb="FF6A7780"/>
-      <sz val="8"/>
-      <name val="Arial"/>
+      <sz val="9"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0E171C"/>
-      <sz val="16"/>
-      <name val="Arial"/>
+      <sz val="17.5"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0E171C"/>
-      <sz val="13"/>
-      <name val="Arial"/>
+      <sz val="14.5"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <color rgb="FF6A7780"/>
-      <sz val="9"/>
-      <name val="Arial"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0A6B74"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF0E171C"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0E171C"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0A6B74"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0A6B74"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF13794A"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FFB42318"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF6A7780"/>
+      <sz val="9.5"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0A6B74"/>
       <sz val="9"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF0E171C"/>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0E171C"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0A6B74"/>
-      <sz val="11"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0A6B74"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF13794A"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FFB42318"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF6A7780"/>
-      <sz val="8.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0A6B74"/>
-      <sz val="8"/>
-      <name val="Arial"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0E171C"/>
-      <sz val="11"/>
-      <name val="Arial"/>
+      <sz val="11.5"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <color rgb="FF6A7780"/>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF6A7780"/>
-      <sz val="9"/>
-      <name val="Arial"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <color rgb="FF0E171C"/>
-      <sz val="8.5"/>
-      <name val="Arial"/>
+      <sz val="9.5"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="9">
@@ -699,7 +708,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -732,12 +741,80 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FFD3D9DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D9DD"/>
+      </right>
       <top style="thin">
         <color rgb="FFD3D9DD"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D9DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D9DD"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D9DD"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD3D9DD"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D9DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D9DD"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD3D9DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D9DD"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD3D9DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD3D9DD"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD3D9DD"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -762,7 +839,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom"/>
@@ -850,21 +927,36 @@
       <alignment wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment indent="1"/>
+      <alignment vertical="bottom" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -894,7 +986,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -930,30 +1022,30 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="3"/>
     </xf>
   </cellXfs>
@@ -1295,7 +1387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1365,16 +1457,16 @@
       <c r="D6" s="9">
         <v>378892.57403020735</v>
       </c>
-      <c r="E6" s="9">
-        <v>10524.793723061315</v>
+      <c r="E6" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -1385,12 +1477,12 @@
         <v>10125.568966697625</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1401,12 +1493,12 @@
         <v>7231.354451968464</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
@@ -1416,7 +1508,7 @@
     </row>
     <row r="11" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>6</v>
@@ -1425,10 +1517,10 @@
         <v>8</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>7</v>
@@ -1756,7 +1848,7 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -1766,7 +1858,7 @@
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -1776,1054 +1868,1042 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="30" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B31" s="30"/>
       <c r="C31" s="30"/>
       <c r="D31" s="30" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E31" s="30"/>
       <c r="F31" s="30"/>
     </row>
     <row r="32" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="31" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B32" s="31"/>
       <c r="C32" s="31"/>
       <c r="D32" s="31" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="32" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B33" s="32"/>
       <c r="C33" s="32"/>
       <c r="D33" s="33" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E33" s="33"/>
       <c r="F33" s="33"/>
     </row>
     <row r="34" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="31" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B34" s="31"/>
       <c r="C34" s="31"/>
       <c r="D34" s="31" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B35" s="33"/>
       <c r="C35" s="33"/>
       <c r="D35" s="33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E35" s="33"/>
       <c r="F35" s="33"/>
     </row>
     <row r="36" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="31" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B36" s="31"/>
       <c r="C36" s="31"/>
       <c r="D36" s="31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
     </row>
     <row r="37" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="33" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B37" s="33"/>
       <c r="C37" s="33"/>
       <c r="D37" s="33" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E37" s="33"/>
       <c r="F37" s="33"/>
     </row>
     <row r="38" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="31" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B38" s="31"/>
       <c r="C38" s="31"/>
-      <c r="D38" s="31" t="s">
+      <c r="D38" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="E38" s="34"/>
+      <c r="F38" s="35" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E38" s="31"/>
-      <c r="F38" s="31"/>
-    </row>
-    <row r="39" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="33"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33" t="s">
-        <v>37</v>
-      </c>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-    </row>
-    <row r="40" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B40" s="31"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="E40" s="31"/>
-      <c r="F40" s="31"/>
-    </row>
-    <row r="41" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B41" s="33"/>
-      <c r="C41" s="33"/>
-      <c r="D41" s="33" t="s">
+      <c r="B39" s="36"/>
+      <c r="C39" s="36"/>
+      <c r="D39" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E41" s="33"/>
-      <c r="F41" s="33"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="38" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" s="39"/>
+      <c r="C41" s="39"/>
+      <c r="D41" s="39"/>
+      <c r="E41" s="39"/>
+      <c r="F41" s="39"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" s="40"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="40"/>
+      <c r="F42" s="40"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="34" t="s">
-        <v>40</v>
-      </c>
-      <c r="B43" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="C43" s="35"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="35"/>
-      <c r="F43" s="35"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="36" t="s">
-        <v>42</v>
-      </c>
-      <c r="B44" s="36"/>
-      <c r="C44" s="36" t="s">
+      <c r="A43" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="D44" s="36"/>
-      <c r="E44" s="36" t="s">
+      <c r="B43" s="41"/>
+      <c r="C43" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="F44" s="36"/>
-    </row>
-    <row r="45" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="37" t="s">
+      <c r="D43" s="41"/>
+      <c r="E43" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="B45" s="37"/>
-      <c r="C45" s="37" t="s">
+      <c r="F43" s="41"/>
+    </row>
+    <row r="44" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="D45" s="37"/>
-      <c r="E45" s="37" t="s">
+      <c r="B44" s="42"/>
+      <c r="C44" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="F45" s="37"/>
-    </row>
-    <row r="47" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="12" t="s">
+      <c r="D44" s="42"/>
+      <c r="E44" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="B47" s="12" t="s">
+      <c r="F44" s="42"/>
+    </row>
+    <row r="46" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="13" t="s">
+      <c r="B46" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="F47" s="13" t="s">
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="13" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="38" t="s">
+      <c r="F46" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B48" s="39" t="s">
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="C48" s="39"/>
-      <c r="D48" s="39"/>
-      <c r="E48" s="40">
+      <c r="B47" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="C47" s="44"/>
+      <c r="D47" s="44"/>
+      <c r="E47" s="45">
         <v>73728.71209883725</v>
       </c>
-      <c r="F48" s="40">
+      <c r="F47" s="45">
         <v>70904.8077475456</v>
       </c>
     </row>
-    <row r="50" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B50" s="12"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="13" t="s">
+    <row r="49" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E50" s="13" t="s">
+      <c r="B49" s="12"/>
+      <c r="C49" s="12"/>
+      <c r="D49" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F50" s="13" t="s">
+      <c r="E49" s="13" t="s">
         <v>57</v>
       </c>
+      <c r="F49" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50" s="46"/>
+      <c r="C50" s="46"/>
+      <c r="D50" s="9">
+        <v>630</v>
+      </c>
+      <c r="E50" s="9">
+        <v>7560</v>
+      </c>
+      <c r="F50" s="9">
+        <v>3780</v>
+      </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="41" t="s">
-        <v>58</v>
-      </c>
-      <c r="B51" s="41"/>
-      <c r="C51" s="41"/>
-      <c r="D51" s="9">
-        <v>630</v>
-      </c>
-      <c r="E51" s="9">
-        <v>7560</v>
-      </c>
-      <c r="F51" s="9">
-        <v>3780</v>
+      <c r="A51" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="47">
+        <v>720</v>
+      </c>
+      <c r="E51" s="47">
+        <v>8640</v>
+      </c>
+      <c r="F51" s="47">
+        <v>4320</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="42">
-        <v>720</v>
-      </c>
-      <c r="E52" s="42">
-        <v>8640</v>
-      </c>
-      <c r="F52" s="42">
-        <v>4320</v>
+      <c r="A52" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="B52" s="46"/>
+      <c r="C52" s="46"/>
+      <c r="D52" s="9">
+        <v>810</v>
+      </c>
+      <c r="E52" s="9">
+        <v>9720</v>
+      </c>
+      <c r="F52" s="9">
+        <v>4860</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="41" t="s">
-        <v>60</v>
-      </c>
-      <c r="B53" s="41"/>
-      <c r="C53" s="41"/>
-      <c r="D53" s="9">
-        <v>810</v>
-      </c>
-      <c r="E53" s="9">
-        <v>9720</v>
-      </c>
-      <c r="F53" s="9">
-        <v>4860</v>
+      <c r="A53" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="47">
+        <v>900</v>
+      </c>
+      <c r="E53" s="47">
+        <v>10800</v>
+      </c>
+      <c r="F53" s="47">
+        <v>5400</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
-      <c r="D54" s="42">
-        <v>900</v>
-      </c>
-      <c r="E54" s="42">
-        <v>10800</v>
-      </c>
-      <c r="F54" s="42">
-        <v>5400</v>
+      <c r="D54" s="47">
+        <v>990</v>
+      </c>
+      <c r="E54" s="47">
+        <v>11880</v>
+      </c>
+      <c r="F54" s="47">
+        <v>5940</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
-      <c r="D55" s="42">
-        <v>990</v>
-      </c>
-      <c r="E55" s="42">
-        <v>11880</v>
-      </c>
-      <c r="F55" s="42">
-        <v>5940</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B56" s="8"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="42">
+      <c r="D55" s="47">
         <v>1080</v>
       </c>
-      <c r="E56" s="42">
+      <c r="E55" s="47">
         <v>12960</v>
       </c>
-      <c r="F56" s="42">
+      <c r="F55" s="47">
         <v>6480</v>
       </c>
     </row>
-    <row r="58" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="43" t="s">
+    <row r="57" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="48" t="s">
+        <v>65</v>
+      </c>
+      <c r="B57" s="48"/>
+      <c r="C57" s="48"/>
+      <c r="D57" s="48"/>
+      <c r="E57" s="48"/>
+      <c r="F57" s="48"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="49" t="s">
+        <v>66</v>
+      </c>
+      <c r="B58" s="49"/>
+      <c r="C58" s="49"/>
+      <c r="D58" s="49"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="49"/>
+    </row>
+    <row r="60" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B60" s="11"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="11"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="50" t="s">
+        <v>68</v>
+      </c>
+      <c r="B61" s="50"/>
+      <c r="C61" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="D61" s="51"/>
+      <c r="E61" s="51"/>
+      <c r="F61" s="51"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="B62" s="50"/>
+      <c r="C62" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="D62" s="51"/>
+      <c r="E62" s="51"/>
+      <c r="F62" s="51"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="50" t="s">
+        <v>72</v>
+      </c>
+      <c r="B63" s="50"/>
+      <c r="C63" s="51" t="s">
+        <v>73</v>
+      </c>
+      <c r="D63" s="51"/>
+      <c r="E63" s="51"/>
+      <c r="F63" s="51"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="50" t="s">
+        <v>74</v>
+      </c>
+      <c r="B64" s="50"/>
+      <c r="C64" s="51" t="s">
+        <v>75</v>
+      </c>
+      <c r="D64" s="51"/>
+      <c r="E64" s="51"/>
+      <c r="F64" s="51"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B65" s="50"/>
+      <c r="C65" s="51" t="s">
+        <v>77</v>
+      </c>
+      <c r="D65" s="51"/>
+      <c r="E65" s="51"/>
+      <c r="F65" s="51"/>
+    </row>
+    <row r="67" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B67" s="11"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="11"/>
+      <c r="E67" s="11"/>
+      <c r="F67" s="11"/>
+    </row>
+    <row r="68" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B68" s="6"/>
+      <c r="C68" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="52" t="s">
+        <v>82</v>
+      </c>
+      <c r="B69" s="52"/>
+      <c r="C69" s="53" t="s">
+        <v>83</v>
+      </c>
+      <c r="D69" s="53"/>
+      <c r="E69" s="53"/>
+      <c r="F69" s="54">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="55" t="s">
+        <v>84</v>
+      </c>
+      <c r="B70" s="55"/>
+      <c r="C70" s="56" t="s">
+        <v>85</v>
+      </c>
+      <c r="D70" s="56"/>
+      <c r="E70" s="56"/>
+      <c r="F70" s="57">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="B71" s="52"/>
+      <c r="C71" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="D71" s="53"/>
+      <c r="E71" s="53"/>
+      <c r="F71" s="54">
+        <v>21.0606</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="55" t="s">
+        <v>88</v>
+      </c>
+      <c r="B72" s="55"/>
+      <c r="C72" s="56" t="s">
+        <v>89</v>
+      </c>
+      <c r="D72" s="56"/>
+      <c r="E72" s="56"/>
+      <c r="F72" s="57">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="52" t="s">
+        <v>90</v>
+      </c>
+      <c r="B73" s="52"/>
+      <c r="C73" s="53" t="s">
+        <v>91</v>
+      </c>
+      <c r="D73" s="53"/>
+      <c r="E73" s="53"/>
+      <c r="F73" s="58">
+        <v>4020</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="55" t="s">
+        <v>92</v>
+      </c>
+      <c r="B74" s="55"/>
+      <c r="C74" s="56" t="s">
+        <v>93</v>
+      </c>
+      <c r="D74" s="56"/>
+      <c r="E74" s="56"/>
+      <c r="F74" s="57">
         <v>64</v>
       </c>
-      <c r="B58" s="43"/>
-      <c r="C58" s="43"/>
-      <c r="D58" s="43"/>
-      <c r="E58" s="43"/>
-      <c r="F58" s="43"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="44" t="s">
-        <v>65</v>
-      </c>
-      <c r="B59" s="44"/>
-      <c r="C59" s="44"/>
-      <c r="D59" s="44"/>
-      <c r="E59" s="44"/>
-      <c r="F59" s="44"/>
-    </row>
-    <row r="61" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="11"/>
-      <c r="F61" s="11"/>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="B62" s="45"/>
-      <c r="C62" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="D62" s="46"/>
-      <c r="E62" s="46"/>
-      <c r="F62" s="46"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="45" t="s">
-        <v>69</v>
-      </c>
-      <c r="B63" s="45"/>
-      <c r="C63" s="46" t="s">
-        <v>70</v>
-      </c>
-      <c r="D63" s="46"/>
-      <c r="E63" s="46"/>
-      <c r="F63" s="46"/>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="45" t="s">
-        <v>71</v>
-      </c>
-      <c r="B64" s="45"/>
-      <c r="C64" s="46" t="s">
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="52" t="s">
+        <v>24</v>
+      </c>
+      <c r="B75" s="52"/>
+      <c r="C75" s="53" t="s">
+        <v>94</v>
+      </c>
+      <c r="D75" s="53"/>
+      <c r="E75" s="53"/>
+      <c r="F75" s="59">
+        <v>199862.17016799998</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="55" t="s">
+        <v>95</v>
+      </c>
+      <c r="B76" s="55"/>
+      <c r="C76" s="56" t="s">
+        <v>96</v>
+      </c>
+      <c r="D76" s="56"/>
+      <c r="E76" s="56"/>
+      <c r="F76" s="60">
+        <v>4542.6</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="52" t="s">
+        <v>97</v>
+      </c>
+      <c r="B77" s="52"/>
+      <c r="C77" s="53" t="s">
+        <v>98</v>
+      </c>
+      <c r="D77" s="53"/>
+      <c r="E77" s="53"/>
+      <c r="F77" s="59">
+        <v>8320</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="55" t="s">
+        <v>45</v>
+      </c>
+      <c r="B78" s="55"/>
+      <c r="C78" s="56" t="s">
+        <v>99</v>
+      </c>
+      <c r="D78" s="56"/>
+      <c r="E78" s="56"/>
+      <c r="F78" s="60">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="52" t="s">
+        <v>100</v>
+      </c>
+      <c r="B79" s="52"/>
+      <c r="C79" s="53" t="s">
+        <v>101</v>
+      </c>
+      <c r="D79" s="53"/>
+      <c r="E79" s="53"/>
+      <c r="F79" s="59">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="55" t="s">
+        <v>102</v>
+      </c>
+      <c r="B80" s="55"/>
+      <c r="C80" s="56" t="s">
+        <v>103</v>
+      </c>
+      <c r="D80" s="56"/>
+      <c r="E80" s="56"/>
+      <c r="F80" s="60">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="52" t="s">
+        <v>104</v>
+      </c>
+      <c r="B81" s="52"/>
+      <c r="C81" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D81" s="53"/>
+      <c r="E81" s="53"/>
+      <c r="F81" s="59">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="55" t="s">
+        <v>106</v>
+      </c>
+      <c r="B82" s="55"/>
+      <c r="C82" s="56" t="s">
+        <v>107</v>
+      </c>
+      <c r="D82" s="56"/>
+      <c r="E82" s="56"/>
+      <c r="F82" s="60">
+        <v>7037.4975</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="B83" s="52"/>
+      <c r="C83" s="53" t="s">
+        <v>108</v>
+      </c>
+      <c r="D83" s="53"/>
+      <c r="E83" s="53"/>
+      <c r="F83" s="59">
+        <v>14850</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="55" t="s">
+        <v>109</v>
+      </c>
+      <c r="B84" s="55"/>
+      <c r="C84" s="56" t="s">
+        <v>110</v>
+      </c>
+      <c r="D84" s="56"/>
+      <c r="E84" s="56"/>
+      <c r="F84" s="60">
+        <v>2567.727</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="61" t="s">
+        <v>111</v>
+      </c>
+      <c r="B85" s="61"/>
+      <c r="C85" s="62" t="s">
+        <v>112</v>
+      </c>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
+      <c r="F85" s="63">
+        <v>247529.994668</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="55" t="s">
+        <v>113</v>
+      </c>
+      <c r="B86" s="55"/>
+      <c r="C86" s="56" t="s">
+        <v>114</v>
+      </c>
+      <c r="D86" s="56"/>
+      <c r="E86" s="56"/>
+      <c r="F86" s="60">
+        <v>1852.8771403200583</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="52" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87" s="52"/>
+      <c r="C87" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="D87" s="53"/>
+      <c r="E87" s="53"/>
+      <c r="F87" s="59">
+        <v>9660.145867493897</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="55" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88" s="55"/>
+      <c r="C88" s="56" t="s">
+        <v>118</v>
+      </c>
+      <c r="D88" s="56"/>
+      <c r="E88" s="56"/>
+      <c r="F88" s="60">
+        <v>100738.95131837211</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="52" t="s">
+        <v>119</v>
+      </c>
+      <c r="B89" s="52"/>
+      <c r="C89" s="53" t="s">
+        <v>120</v>
+      </c>
+      <c r="D89" s="53"/>
+      <c r="E89" s="53"/>
+      <c r="F89" s="59">
+        <v>110399.097185866</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="55" t="s">
+        <v>121</v>
+      </c>
+      <c r="B90" s="55"/>
+      <c r="C90" s="56" t="s">
+        <v>122</v>
+      </c>
+      <c r="D90" s="56"/>
+      <c r="E90" s="56"/>
+      <c r="F90" s="60">
+        <v>19110.605036021243</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" s="61" t="s">
+        <v>123</v>
+      </c>
+      <c r="B91" s="61"/>
+      <c r="C91" s="62" t="s">
+        <v>124</v>
+      </c>
+      <c r="D91" s="62"/>
+      <c r="E91" s="62"/>
+      <c r="F91" s="63">
+        <v>378892.57403020735</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="61" t="s">
+        <v>125</v>
+      </c>
+      <c r="B92" s="61"/>
+      <c r="C92" s="62" t="s">
+        <v>126</v>
+      </c>
+      <c r="D92" s="62"/>
+      <c r="E92" s="62"/>
+      <c r="F92" s="63">
+        <v>268493.4768443414</v>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B94" s="11"/>
+      <c r="C94" s="11"/>
+      <c r="D94" s="11"/>
+      <c r="E94" s="11"/>
+      <c r="F94" s="11"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="B95" s="50"/>
+      <c r="C95" s="51" t="s">
+        <v>129</v>
+      </c>
+      <c r="D95" s="51"/>
+      <c r="E95" s="51"/>
+      <c r="F95" s="51"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="B96" s="50"/>
+      <c r="C96" s="51" t="s">
+        <v>131</v>
+      </c>
+      <c r="D96" s="51"/>
+      <c r="E96" s="51"/>
+      <c r="F96" s="51"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="B97" s="50"/>
+      <c r="C97" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="D97" s="51"/>
+      <c r="E97" s="51"/>
+      <c r="F97" s="51"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" s="50" t="s">
+        <v>134</v>
+      </c>
+      <c r="B98" s="50"/>
+      <c r="C98" s="51" t="s">
+        <v>135</v>
+      </c>
+      <c r="D98" s="51"/>
+      <c r="E98" s="51"/>
+      <c r="F98" s="51"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" s="50" t="s">
+        <v>136</v>
+      </c>
+      <c r="B99" s="50"/>
+      <c r="C99" s="51" t="s">
+        <v>137</v>
+      </c>
+      <c r="D99" s="51"/>
+      <c r="E99" s="51"/>
+      <c r="F99" s="51"/>
+    </row>
+    <row r="101" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" s="48" t="s">
+        <v>138</v>
+      </c>
+      <c r="B101" s="48"/>
+      <c r="C101" s="48"/>
+      <c r="D101" s="48"/>
+      <c r="E101" s="48"/>
+      <c r="F101" s="48"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" s="49" t="s">
+        <v>139</v>
+      </c>
+      <c r="B102" s="49"/>
+      <c r="C102" s="49"/>
+      <c r="D102" s="49"/>
+      <c r="E102" s="49"/>
+      <c r="F102" s="49"/>
+    </row>
+    <row r="104" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" s="64" t="s">
+        <v>44</v>
+      </c>
+      <c r="B104" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="C104" s="66" t="s">
+        <v>140</v>
+      </c>
+      <c r="D104" s="66"/>
+      <c r="E104" s="66"/>
+      <c r="F104" s="67" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="105" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" s="68" t="s">
+        <v>142</v>
+      </c>
+      <c r="B105" s="69">
+        <v>130</v>
+      </c>
+      <c r="C105" s="66" t="s">
+        <v>143</v>
+      </c>
+      <c r="D105" s="66"/>
+      <c r="E105" s="66"/>
+      <c r="F105" s="67" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="106" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" s="68" t="s">
+        <v>145</v>
+      </c>
+      <c r="B106" s="69">
+        <v>45</v>
+      </c>
+      <c r="C106" s="66" t="s">
+        <v>146</v>
+      </c>
+      <c r="D106" s="66"/>
+      <c r="E106" s="66"/>
+      <c r="F106" s="67" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="107" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="B107" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="C107" s="66" t="s">
+        <v>149</v>
+      </c>
+      <c r="D107" s="66"/>
+      <c r="E107" s="66"/>
+      <c r="F107" s="67" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="108" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" s="68" t="s">
+        <v>151</v>
+      </c>
+      <c r="B108" s="70" t="s">
+        <v>152</v>
+      </c>
+      <c r="C108" s="66" t="s">
+        <v>153</v>
+      </c>
+      <c r="D108" s="66"/>
+      <c r="E108" s="66"/>
+      <c r="F108" s="67" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="109" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" s="64" t="s">
+        <v>155</v>
+      </c>
+      <c r="B109" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="C109" s="66" t="s">
+        <v>156</v>
+      </c>
+      <c r="D109" s="66"/>
+      <c r="E109" s="66"/>
+      <c r="F109" s="67" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="110" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" s="68" t="s">
         <v>72</v>
       </c>
-      <c r="D64" s="46"/>
-      <c r="E64" s="46"/>
-      <c r="F64" s="46"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="45" t="s">
-        <v>73</v>
-      </c>
-      <c r="B65" s="45"/>
-      <c r="C65" s="46" t="s">
-        <v>74</v>
-      </c>
-      <c r="D65" s="46"/>
-      <c r="E65" s="46"/>
-      <c r="F65" s="46"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="45" t="s">
-        <v>75</v>
-      </c>
-      <c r="B66" s="45"/>
-      <c r="C66" s="46" t="s">
-        <v>76</v>
-      </c>
-      <c r="D66" s="46"/>
-      <c r="E66" s="46"/>
-      <c r="F66" s="46"/>
-    </row>
-    <row r="68" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="B68" s="11"/>
-      <c r="C68" s="11"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="11"/>
-      <c r="F68" s="11"/>
-    </row>
-    <row r="69" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B69" s="6"/>
-      <c r="C69" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="D69" s="6"/>
-      <c r="E69" s="6"/>
-      <c r="F69" s="7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="47" t="s">
-        <v>81</v>
-      </c>
-      <c r="B70" s="47"/>
-      <c r="C70" s="48" t="s">
-        <v>82</v>
-      </c>
-      <c r="D70" s="48"/>
-      <c r="E70" s="48"/>
-      <c r="F70" s="49">
+      <c r="B110" s="70" t="s">
+        <v>158</v>
+      </c>
+      <c r="C110" s="66" t="s">
+        <v>159</v>
+      </c>
+      <c r="D110" s="66"/>
+      <c r="E110" s="66"/>
+      <c r="F110" s="67" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="111" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" s="64" t="s">
+        <v>160</v>
+      </c>
+      <c r="B111" s="65" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="50" t="s">
-        <v>83</v>
-      </c>
-      <c r="B71" s="50"/>
-      <c r="C71" s="51" t="s">
-        <v>84</v>
-      </c>
-      <c r="D71" s="51"/>
-      <c r="E71" s="51"/>
-      <c r="F71" s="52">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="47" t="s">
-        <v>85</v>
-      </c>
-      <c r="B72" s="47"/>
-      <c r="C72" s="48" t="s">
-        <v>86</v>
-      </c>
-      <c r="D72" s="48"/>
-      <c r="E72" s="48"/>
-      <c r="F72" s="49">
-        <v>21.0606</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="50" t="s">
-        <v>87</v>
-      </c>
-      <c r="B73" s="50"/>
-      <c r="C73" s="51" t="s">
-        <v>88</v>
-      </c>
-      <c r="D73" s="51"/>
-      <c r="E73" s="51"/>
-      <c r="F73" s="52">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="47" t="s">
-        <v>89</v>
-      </c>
-      <c r="B74" s="47"/>
-      <c r="C74" s="48" t="s">
-        <v>90</v>
-      </c>
-      <c r="D74" s="48"/>
-      <c r="E74" s="48"/>
-      <c r="F74" s="53">
-        <v>4020</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" s="50" t="s">
-        <v>91</v>
-      </c>
-      <c r="B75" s="50"/>
-      <c r="C75" s="51" t="s">
-        <v>92</v>
-      </c>
-      <c r="D75" s="51"/>
-      <c r="E75" s="51"/>
-      <c r="F75" s="52">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" s="47" t="s">
-        <v>23</v>
-      </c>
-      <c r="B76" s="47"/>
-      <c r="C76" s="48" t="s">
-        <v>93</v>
-      </c>
-      <c r="D76" s="48"/>
-      <c r="E76" s="48"/>
-      <c r="F76" s="54">
-        <v>199862.17016799998</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" s="50" t="s">
-        <v>94</v>
-      </c>
-      <c r="B77" s="50"/>
-      <c r="C77" s="51" t="s">
-        <v>95</v>
-      </c>
-      <c r="D77" s="51"/>
-      <c r="E77" s="51"/>
-      <c r="F77" s="55">
-        <v>4542.6</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A78" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B78" s="47"/>
-      <c r="C78" s="48" t="s">
-        <v>97</v>
-      </c>
-      <c r="D78" s="48"/>
-      <c r="E78" s="48"/>
-      <c r="F78" s="54">
-        <v>8320</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B79" s="50"/>
-      <c r="C79" s="51" t="s">
-        <v>98</v>
-      </c>
-      <c r="D79" s="51"/>
-      <c r="E79" s="51"/>
-      <c r="F79" s="55">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="47" t="s">
-        <v>99</v>
-      </c>
-      <c r="B80" s="47"/>
-      <c r="C80" s="48" t="s">
-        <v>100</v>
-      </c>
-      <c r="D80" s="48"/>
-      <c r="E80" s="48"/>
-      <c r="F80" s="54">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A81" s="50" t="s">
-        <v>101</v>
-      </c>
-      <c r="B81" s="50"/>
-      <c r="C81" s="51" t="s">
-        <v>102</v>
-      </c>
-      <c r="D81" s="51"/>
-      <c r="E81" s="51"/>
-      <c r="F81" s="55">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="B82" s="47"/>
-      <c r="C82" s="48" t="s">
-        <v>104</v>
-      </c>
-      <c r="D82" s="48"/>
-      <c r="E82" s="48"/>
-      <c r="F82" s="54">
-        <v>1650</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A83" s="50" t="s">
-        <v>105</v>
-      </c>
-      <c r="B83" s="50"/>
-      <c r="C83" s="51" t="s">
-        <v>106</v>
-      </c>
-      <c r="D83" s="51"/>
-      <c r="E83" s="51"/>
-      <c r="F83" s="55">
-        <v>7037.4975</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A84" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="B84" s="47"/>
-      <c r="C84" s="48" t="s">
-        <v>107</v>
-      </c>
-      <c r="D84" s="48"/>
-      <c r="E84" s="48"/>
-      <c r="F84" s="54">
-        <v>14850</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A85" s="50" t="s">
-        <v>108</v>
-      </c>
-      <c r="B85" s="50"/>
-      <c r="C85" s="51" t="s">
-        <v>109</v>
-      </c>
-      <c r="D85" s="51"/>
-      <c r="E85" s="51"/>
-      <c r="F85" s="55">
-        <v>2567.727</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A86" s="56" t="s">
-        <v>110</v>
-      </c>
-      <c r="B86" s="56"/>
-      <c r="C86" s="57" t="s">
-        <v>111</v>
-      </c>
-      <c r="D86" s="57"/>
-      <c r="E86" s="57"/>
-      <c r="F86" s="58">
-        <v>247529.994668</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A87" s="50" t="s">
-        <v>112</v>
-      </c>
-      <c r="B87" s="50"/>
-      <c r="C87" s="51" t="s">
-        <v>113</v>
-      </c>
-      <c r="D87" s="51"/>
-      <c r="E87" s="51"/>
-      <c r="F87" s="55">
-        <v>1852.8771403200583</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A88" s="47" t="s">
-        <v>114</v>
-      </c>
-      <c r="B88" s="47"/>
-      <c r="C88" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="D88" s="48"/>
-      <c r="E88" s="48"/>
-      <c r="F88" s="54">
-        <v>9660.145867493897</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A89" s="50" t="s">
-        <v>116</v>
-      </c>
-      <c r="B89" s="50"/>
-      <c r="C89" s="51" t="s">
-        <v>117</v>
-      </c>
-      <c r="D89" s="51"/>
-      <c r="E89" s="51"/>
-      <c r="F89" s="55">
-        <v>100738.95131837211</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A90" s="47" t="s">
-        <v>118</v>
-      </c>
-      <c r="B90" s="47"/>
-      <c r="C90" s="48" t="s">
-        <v>119</v>
-      </c>
-      <c r="D90" s="48"/>
-      <c r="E90" s="48"/>
-      <c r="F90" s="54">
-        <v>110399.097185866</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A91" s="50" t="s">
-        <v>120</v>
-      </c>
-      <c r="B91" s="50"/>
-      <c r="C91" s="51" t="s">
-        <v>121</v>
-      </c>
-      <c r="D91" s="51"/>
-      <c r="E91" s="51"/>
-      <c r="F91" s="55">
-        <v>19110.605036021243</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A92" s="56" t="s">
-        <v>122</v>
-      </c>
-      <c r="B92" s="56"/>
-      <c r="C92" s="57" t="s">
-        <v>123</v>
-      </c>
-      <c r="D92" s="57"/>
-      <c r="E92" s="57"/>
-      <c r="F92" s="58">
-        <v>378892.57403020735</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A93" s="56" t="s">
-        <v>124</v>
-      </c>
-      <c r="B93" s="56"/>
-      <c r="C93" s="57" t="s">
-        <v>125</v>
-      </c>
-      <c r="D93" s="57"/>
-      <c r="E93" s="57"/>
-      <c r="F93" s="58">
-        <v>268493.4768443414</v>
-      </c>
-    </row>
-    <row r="95" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A95" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="B95" s="11"/>
-      <c r="C95" s="11"/>
-      <c r="D95" s="11"/>
-      <c r="E95" s="11"/>
-      <c r="F95" s="11"/>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A96" s="45" t="s">
-        <v>127</v>
-      </c>
-      <c r="B96" s="45"/>
-      <c r="C96" s="46" t="s">
-        <v>128</v>
-      </c>
-      <c r="D96" s="46"/>
-      <c r="E96" s="46"/>
-      <c r="F96" s="46"/>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A97" s="45" t="s">
-        <v>129</v>
-      </c>
-      <c r="B97" s="45"/>
-      <c r="C97" s="46" t="s">
-        <v>130</v>
-      </c>
-      <c r="D97" s="46"/>
-      <c r="E97" s="46"/>
-      <c r="F97" s="46"/>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A98" s="45" t="s">
-        <v>131</v>
-      </c>
-      <c r="B98" s="45"/>
-      <c r="C98" s="46" t="s">
-        <v>132</v>
-      </c>
-      <c r="D98" s="46"/>
-      <c r="E98" s="46"/>
-      <c r="F98" s="46"/>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A99" s="45" t="s">
-        <v>133</v>
-      </c>
-      <c r="B99" s="45"/>
-      <c r="C99" s="46" t="s">
-        <v>134</v>
-      </c>
-      <c r="D99" s="46"/>
-      <c r="E99" s="46"/>
-      <c r="F99" s="46"/>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A100" s="45" t="s">
-        <v>135</v>
-      </c>
-      <c r="B100" s="45"/>
-      <c r="C100" s="46" t="s">
-        <v>136</v>
-      </c>
-      <c r="D100" s="46"/>
-      <c r="E100" s="46"/>
-      <c r="F100" s="46"/>
-    </row>
-    <row r="102" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A102" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B102" s="43"/>
-      <c r="C102" s="43"/>
-      <c r="D102" s="43"/>
-      <c r="E102" s="43"/>
-      <c r="F102" s="43"/>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A103" s="44" t="s">
-        <v>138</v>
-      </c>
-      <c r="B103" s="44"/>
-      <c r="C103" s="44"/>
-      <c r="D103" s="44"/>
-      <c r="E103" s="44"/>
-      <c r="F103" s="44"/>
-    </row>
-    <row r="105" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A105" s="59" t="s">
-        <v>43</v>
-      </c>
-      <c r="B105" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="C105" s="61" t="s">
-        <v>139</v>
-      </c>
-      <c r="D105" s="61"/>
-      <c r="E105" s="61"/>
-      <c r="F105" s="62" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="106" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A106" s="63" t="s">
-        <v>141</v>
-      </c>
-      <c r="B106" s="64">
-        <v>130</v>
-      </c>
-      <c r="C106" s="61" t="s">
-        <v>142</v>
-      </c>
-      <c r="D106" s="61"/>
-      <c r="E106" s="61"/>
-      <c r="F106" s="62" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="107" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A107" s="63" t="s">
-        <v>144</v>
-      </c>
-      <c r="B107" s="64">
-        <v>45</v>
-      </c>
-      <c r="C107" s="61" t="s">
-        <v>145</v>
-      </c>
-      <c r="D107" s="61"/>
-      <c r="E107" s="61"/>
-      <c r="F107" s="62" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="108" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A108" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="B108" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="C108" s="61" t="s">
-        <v>148</v>
-      </c>
-      <c r="D108" s="61"/>
-      <c r="E108" s="61"/>
-      <c r="F108" s="62" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="109" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A109" s="63" t="s">
-        <v>150</v>
-      </c>
-      <c r="B109" s="65" t="s">
-        <v>151</v>
-      </c>
-      <c r="C109" s="61" t="s">
-        <v>152</v>
-      </c>
-      <c r="D109" s="61"/>
-      <c r="E109" s="61"/>
-      <c r="F109" s="62" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="110" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A110" s="59" t="s">
-        <v>154</v>
-      </c>
-      <c r="B110" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="C110" s="61" t="s">
-        <v>155</v>
-      </c>
-      <c r="D110" s="61"/>
-      <c r="E110" s="61"/>
-      <c r="F110" s="62" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="111" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A111" s="63" t="s">
-        <v>71</v>
-      </c>
-      <c r="B111" s="65" t="s">
-        <v>157</v>
-      </c>
-      <c r="C111" s="61" t="s">
-        <v>158</v>
-      </c>
-      <c r="D111" s="61"/>
-      <c r="E111" s="61"/>
-      <c r="F111" s="62" t="s">
-        <v>156</v>
+      <c r="C111" s="66" t="s">
+        <v>161</v>
+      </c>
+      <c r="D111" s="66"/>
+      <c r="E111" s="66"/>
+      <c r="F111" s="67" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="112" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A112" s="59" t="s">
-        <v>159</v>
-      </c>
-      <c r="B112" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="C112" s="61" t="s">
-        <v>160</v>
-      </c>
-      <c r="D112" s="61"/>
-      <c r="E112" s="61"/>
-      <c r="F112" s="62" t="s">
-        <v>161</v>
+      <c r="A112" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="B112" s="70" t="s">
+        <v>164</v>
+      </c>
+      <c r="C112" s="66" t="s">
+        <v>165</v>
+      </c>
+      <c r="D112" s="66"/>
+      <c r="E112" s="66"/>
+      <c r="F112" s="67" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="113" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A113" s="63" t="s">
-        <v>162</v>
-      </c>
-      <c r="B113" s="65" t="s">
-        <v>163</v>
-      </c>
-      <c r="C113" s="61" t="s">
-        <v>164</v>
-      </c>
-      <c r="D113" s="61"/>
-      <c r="E113" s="61"/>
-      <c r="F113" s="62" t="s">
-        <v>165</v>
+      <c r="A113" s="68" t="s">
+        <v>167</v>
+      </c>
+      <c r="B113" s="70" t="s">
+        <v>168</v>
+      </c>
+      <c r="C113" s="71" t="s">
+        <v>169</v>
+      </c>
+      <c r="D113" s="71"/>
+      <c r="E113" s="71"/>
+      <c r="F113" s="65" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="114" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A114" s="63" t="s">
-        <v>166</v>
-      </c>
-      <c r="B114" s="65" t="s">
-        <v>167</v>
+      <c r="A114" s="68" t="s">
+        <v>170</v>
+      </c>
+      <c r="B114" s="70" t="s">
+        <v>171</v>
       </c>
       <c r="C114" s="66" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D114" s="66"/>
       <c r="E114" s="66"/>
-      <c r="F114" s="60" t="s">
-        <v>35</v>
+      <c r="F114" s="67" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="115" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A115" s="63" t="s">
-        <v>169</v>
-      </c>
-      <c r="B115" s="65" t="s">
-        <v>170</v>
-      </c>
-      <c r="C115" s="61" t="s">
-        <v>171</v>
-      </c>
-      <c r="D115" s="61"/>
-      <c r="E115" s="61"/>
-      <c r="F115" s="62" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="116" ht="13" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A116" s="63" t="s">
-        <v>173</v>
-      </c>
-      <c r="B116" s="65" t="s">
+      <c r="A115" s="68" t="s">
         <v>174</v>
       </c>
-      <c r="C116" t="s">
-        <v>35</v>
-      </c>
-      <c r="D116"/>
-      <c r="E116"/>
-      <c r="F116" t="s">
-        <v>35</v>
+      <c r="B115" s="70" t="s">
+        <v>175</v>
+      </c>
+      <c r="C115" t="s">
+        <v>36</v>
+      </c>
+      <c r="D115"/>
+      <c r="E115"/>
+      <c r="F115" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="139">
+  <mergeCells count="136">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:D2"/>
@@ -2851,32 +2931,31 @@
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="D37:F37"/>
     <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="D38:E38"/>
     <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:F39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:F41"/>
-    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:F43"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="E44:F44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="B46:D46"/>
     <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="A49:C49"/>
     <mergeCell ref="A50:C50"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="A52:C52"/>
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="A54:C54"/>
     <mergeCell ref="A55:C55"/>
-    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="A57:F57"/>
     <mergeCell ref="A58:F58"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="C61:F61"/>
     <mergeCell ref="A62:B62"/>
     <mergeCell ref="C62:F62"/>
     <mergeCell ref="A63:B63"/>
@@ -2885,9 +2964,9 @@
     <mergeCell ref="C64:F64"/>
     <mergeCell ref="A65:B65"/>
     <mergeCell ref="C65:F65"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="C66:F66"/>
-    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="C68:E68"/>
     <mergeCell ref="A69:B69"/>
     <mergeCell ref="C69:E69"/>
     <mergeCell ref="A70:B70"/>
@@ -2936,9 +3015,9 @@
     <mergeCell ref="C91:E91"/>
     <mergeCell ref="A92:B92"/>
     <mergeCell ref="C92:E92"/>
-    <mergeCell ref="A93:B93"/>
-    <mergeCell ref="C93:E93"/>
-    <mergeCell ref="A95:F95"/>
+    <mergeCell ref="A94:F94"/>
+    <mergeCell ref="A95:B95"/>
+    <mergeCell ref="C95:F95"/>
     <mergeCell ref="A96:B96"/>
     <mergeCell ref="C96:F96"/>
     <mergeCell ref="A97:B97"/>
@@ -2947,10 +3026,9 @@
     <mergeCell ref="C98:F98"/>
     <mergeCell ref="A99:B99"/>
     <mergeCell ref="C99:F99"/>
-    <mergeCell ref="A100:B100"/>
-    <mergeCell ref="C100:F100"/>
+    <mergeCell ref="A101:F101"/>
     <mergeCell ref="A102:F102"/>
-    <mergeCell ref="A103:F103"/>
+    <mergeCell ref="C104:E104"/>
     <mergeCell ref="C105:E105"/>
     <mergeCell ref="C106:E106"/>
     <mergeCell ref="C107:E107"/>
@@ -2962,16 +3040,15 @@
     <mergeCell ref="C113:E113"/>
     <mergeCell ref="C114:E114"/>
     <mergeCell ref="C115:E115"/>
-    <mergeCell ref="C116:E116"/>
   </mergeCells>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.55" header="0.25" footer="0.25"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="78" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="82" fitToWidth="1" fitToHeight="1"/>
   <headerFooter>
     <oddFooter>&amp;L&amp;8ul. Kwiatowa 24, Piastów&amp;R&amp;8Strona &amp;P z &amp;N</oddFooter>
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
-    <brk id="57" max="16838" man="1"/>
-    <brk id="101" max="16838" man="1"/>
+    <brk id="56" max="16838" man="1"/>
+    <brk id="100" max="16838" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>